<commit_message>
Initialisation du calculateur réussi
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="381" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{202E8FD5-4A59-41BE-AF4A-58D246F5DC77}"/>
+  <xr:revisionPtr revIDLastSave="384" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18B51A76-C012-4788-B7D5-C75B90B7CC76}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="238">
   <si>
     <t>Montant</t>
   </si>
@@ -749,19 +749,16 @@
     <t>Tantièmes Stationnement</t>
   </si>
   <si>
-    <t>Lots</t>
-  </si>
-  <si>
     <t>Lot 462 - Parking n°64 au -2</t>
   </si>
   <si>
-    <t>IDTantiemes</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
     <t>ID prestation</t>
+  </si>
+  <si>
+    <t>ID tantiemes</t>
   </si>
 </sst>
 </file>
@@ -869,6 +866,351 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1173,351 +1515,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1552,10 +1549,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="BdBudgetPrevisionnel8" displayName="BdBudgetPrevisionnel8" ref="A1:F35" totalsRowCount="1">
   <autoFilter ref="A1:F34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1563,12 +1556,12 @@
     <sortCondition ref="C1:C34"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{3B91602D-BA59-47C1-AD19-EAA938B961C7}" name="IDTantiemes"/>
+    <tableColumn id="1" xr3:uid="{3B91602D-BA59-47C1-AD19-EAA938B961C7}" name="ID tantiemes"/>
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="5" xr3:uid="{94753CD6-8AE2-4955-84AD-F394A68DA3B9}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1578,7 +1571,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}" name="BdCoproprietaires2" displayName="BdCoproprietaires2" ref="A1:P5" totalsRowShown="0">
   <autoFilter ref="A1:P5" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}"/>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Lots" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="49"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
     <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="48">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
@@ -1608,16 +1601,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="31"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="28">
       <calculatedColumnFormula>IF(BdCompetition9[[#This Row],[Taxes]]="TTC",BdCompetition9[[#This Row],[Cout]],BdCompetition9[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1630,16 +1623,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="26">
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="21">
       <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1656,7 +1649,7 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="19" totalsRowDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1669,23 +1662,23 @@
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="24">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="17">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="18"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="17"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="16"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="15"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="11"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="13"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
   </tableColumns>
@@ -1698,7 +1691,7 @@
   <autoFilter ref="A1:D9" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8584E7DE-3397-4839-B3F7-5BE29387C4A6}" name="Label des règles"/>
-    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{4C91DD63-5027-4E87-B95E-BCB801F28C1C}" name="Taxes"/>
     <tableColumn id="4" xr3:uid="{41CB6CC9-60A9-4712-874D-13D61D2EB5DE}" name="Total TTC">
       <calculatedColumnFormula>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</calculatedColumnFormula>
@@ -1713,7 +1706,7 @@
   <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1998,10 +1991,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C1" t="s">
         <v>114</v>
@@ -2712,7 +2705,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
         <v>164</v>
@@ -2865,7 +2858,7 @@
         <v>462</v>
       </c>
       <c r="B5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C5" s="10">
         <v>7</v>
@@ -2924,7 +2917,7 @@
         <v>113</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D1" t="s">
         <v>112</v>

</xml_diff>

<commit_message>
Intégration du calcul des charge selon température
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="384" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18B51A76-C012-4788-B7D5-C75B90B7CC76}"/>
+  <xr:revisionPtr revIDLastSave="398" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD57C84B-8071-43E9-B1D5-8EE826D5B0A1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="240">
   <si>
     <t>Montant</t>
   </si>
@@ -759,6 +759,12 @@
   </si>
   <si>
     <t>ID tantiemes</t>
+  </si>
+  <si>
+    <t>Top consommation chauffage</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -846,9 +852,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="50">
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1266,24 +1269,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1536,6 +1521,27 @@
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1550,18 +1556,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="BdBudgetPrevisionnel8" displayName="BdBudgetPrevisionnel8" ref="A1:F35" totalsRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="BdBudgetPrevisionnel8" displayName="BdBudgetPrevisionnel8" ref="A1:F34">
   <autoFilter ref="A1:F34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:F34">
-    <sortCondition ref="C1:C34"/>
-  </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3B91602D-BA59-47C1-AD19-EAA938B961C7}" name="ID tantiemes"/>
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
-    <tableColumn id="5" xr3:uid="{94753CD6-8AE2-4955-84AD-F394A68DA3B9}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{2D489B7F-CE46-4597-8866-46E6A31D6BF8}" name="Top consommation chauffage"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1571,24 +1574,24 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}" name="BdCoproprietaires2" displayName="BdCoproprietaires2" ref="A1:P5" totalsRowShown="0">
   <autoFilter ref="A1:P5" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}"/>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="47"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="48">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="46">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="45"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="44"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="43"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="42"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="41"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="40"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="39"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="38"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="37"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="42"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="41"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="40"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="39"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="38"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="37"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="36"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="35"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1596,21 +1599,27 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="BdCompetition9" displayName="BdCompetition9" ref="A1:H47" totalsRowShown="0">
-  <autoFilter ref="A1:H47" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
+  <autoFilter ref="A1:H47" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Fourniture de granulé de bois"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H47">
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="30"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="28">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="27">
       <calculatedColumnFormula>IF(BdCompetition9[[#This Row],[Taxes]]="TTC",BdCompetition9[[#This Row],[Cout]],BdCompetition9[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1623,16 +1632,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="23"/>
     <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="21">
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="20">
       <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1649,7 +1658,7 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="18" totalsRowDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1662,23 +1671,23 @@
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="17">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="16">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="13"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="12"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="10"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="8"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="7"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="6"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="4"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="10"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="9"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="8"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="5"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
   </tableColumns>
@@ -1691,7 +1700,7 @@
   <autoFilter ref="A1:D9" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8584E7DE-3397-4839-B3F7-5BE29387C4A6}" name="Label des règles"/>
-    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{4C91DD63-5027-4E87-B95E-BCB801F28C1C}" name="Taxes"/>
     <tableColumn id="4" xr3:uid="{41CB6CC9-60A9-4712-874D-13D61D2EB5DE}" name="Total TTC">
       <calculatedColumnFormula>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</calculatedColumnFormula>
@@ -1706,7 +1715,7 @@
   <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1978,15 +1987,15 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="42.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1997,16 +2006,16 @@
         <v>235</v>
       </c>
       <c r="C1" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="D1" t="s">
-        <v>164</v>
-      </c>
-      <c r="E1" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>117</v>
+      </c>
+      <c r="F1" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -2017,15 +2026,12 @@
         <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>194</v>
       </c>
       <c r="D2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E2" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="1">
+      <c r="E2" s="1">
         <v>1500</v>
       </c>
     </row>
@@ -2037,15 +2043,12 @@
         <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>195</v>
       </c>
       <c r="D3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E3" t="s">
         <v>100</v>
       </c>
-      <c r="F3" s="1">
+      <c r="E3" s="1">
         <v>1500</v>
       </c>
     </row>
@@ -2057,15 +2060,12 @@
         <v>191</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>198</v>
       </c>
       <c r="D4" t="s">
         <v>198</v>
       </c>
-      <c r="E4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F4" s="1">
+      <c r="E4" s="1">
         <v>2000</v>
       </c>
     </row>
@@ -2077,15 +2077,12 @@
         <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>196</v>
       </c>
       <c r="D5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E5" t="s">
         <v>102</v>
       </c>
-      <c r="F5" s="1">
+      <c r="E5" s="1">
         <v>2900</v>
       </c>
     </row>
@@ -2097,15 +2094,12 @@
         <v>192</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>199</v>
       </c>
       <c r="D6" t="s">
         <v>199</v>
       </c>
-      <c r="E6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F6" s="1">
+      <c r="E6" s="1">
         <v>1000</v>
       </c>
     </row>
@@ -2117,15 +2111,12 @@
         <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>197</v>
       </c>
       <c r="D7" t="s">
-        <v>197</v>
-      </c>
-      <c r="E7" t="s">
         <v>103</v>
       </c>
-      <c r="F7" s="1">
+      <c r="E7" s="1">
         <v>2900</v>
       </c>
     </row>
@@ -2137,15 +2128,12 @@
         <v>193</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>200</v>
       </c>
       <c r="D8" t="s">
         <v>200</v>
       </c>
-      <c r="E8" t="s">
-        <v>200</v>
-      </c>
-      <c r="F8" s="1">
+      <c r="E8" s="1">
         <v>1000</v>
       </c>
     </row>
@@ -2157,15 +2145,12 @@
         <v>85</v>
       </c>
       <c r="C9" t="s">
-        <v>220</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
         <v>54</v>
       </c>
-      <c r="E9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="1">
+      <c r="E9" s="1">
         <v>750</v>
       </c>
     </row>
@@ -2177,15 +2162,12 @@
         <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>220</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="1">
+      <c r="E10" s="1">
         <v>6200</v>
       </c>
     </row>
@@ -2197,15 +2179,12 @@
         <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>220</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
         <v>50</v>
       </c>
-      <c r="E11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="1">
+      <c r="E11" s="1">
         <v>1050</v>
       </c>
     </row>
@@ -2217,15 +2196,12 @@
         <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>220</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
         <v>49</v>
       </c>
-      <c r="E12" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="1">
+      <c r="E12" s="1">
         <v>900</v>
       </c>
     </row>
@@ -2237,15 +2213,12 @@
         <v>79</v>
       </c>
       <c r="C13" t="s">
-        <v>220</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
         <v>48</v>
       </c>
-      <c r="E13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" s="1">
+      <c r="E13" s="1">
         <v>920</v>
       </c>
     </row>
@@ -2257,15 +2230,12 @@
         <v>72</v>
       </c>
       <c r="C14" t="s">
-        <v>220</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
         <v>41</v>
       </c>
-      <c r="E14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="1">
+      <c r="E14" s="1">
         <v>35000</v>
       </c>
     </row>
@@ -2277,15 +2247,12 @@
         <v>73</v>
       </c>
       <c r="C15" t="s">
-        <v>220</v>
+        <v>124</v>
       </c>
       <c r="D15" t="s">
-        <v>124</v>
-      </c>
-      <c r="E15" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="1">
+      <c r="E15" s="1">
         <v>1500</v>
       </c>
     </row>
@@ -2297,15 +2264,12 @@
         <v>82</v>
       </c>
       <c r="C16" t="s">
-        <v>220</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
         <v>51</v>
       </c>
-      <c r="E16" t="s">
-        <v>51</v>
-      </c>
-      <c r="F16" s="1">
+      <c r="E16" s="1">
         <v>580</v>
       </c>
     </row>
@@ -2317,15 +2281,12 @@
         <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>220</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
         <v>56</v>
       </c>
-      <c r="E17" t="s">
-        <v>56</v>
-      </c>
-      <c r="F17" s="1">
+      <c r="E17" s="1">
         <v>570</v>
       </c>
     </row>
@@ -2337,15 +2298,12 @@
         <v>88</v>
       </c>
       <c r="C18" t="s">
-        <v>220</v>
+        <v>57</v>
       </c>
       <c r="D18" t="s">
         <v>57</v>
       </c>
-      <c r="E18" t="s">
-        <v>57</v>
-      </c>
-      <c r="F18" s="1">
+      <c r="E18" s="1">
         <v>850</v>
       </c>
     </row>
@@ -2357,15 +2315,12 @@
         <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>220</v>
+        <v>46</v>
       </c>
       <c r="D19" t="s">
         <v>46</v>
       </c>
-      <c r="E19" t="s">
-        <v>46</v>
-      </c>
-      <c r="F19" s="1">
+      <c r="E19" s="1">
         <v>240</v>
       </c>
     </row>
@@ -2377,15 +2332,12 @@
         <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>220</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
         <v>45</v>
       </c>
-      <c r="E20" t="s">
-        <v>45</v>
-      </c>
-      <c r="F20" s="1">
+      <c r="E20" s="1">
         <v>220</v>
       </c>
     </row>
@@ -2397,15 +2349,12 @@
         <v>74</v>
       </c>
       <c r="C21" t="s">
-        <v>220</v>
+        <v>43</v>
       </c>
       <c r="D21" t="s">
         <v>43</v>
       </c>
-      <c r="E21" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="1">
+      <c r="E21" s="1">
         <v>18000</v>
       </c>
     </row>
@@ -2417,15 +2366,12 @@
         <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>220</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
         <v>47</v>
       </c>
-      <c r="E22" t="s">
-        <v>47</v>
-      </c>
-      <c r="F22" s="1"/>
+      <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -2435,15 +2381,12 @@
         <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>220</v>
+        <v>44</v>
       </c>
       <c r="D23" t="s">
         <v>44</v>
       </c>
-      <c r="E23" t="s">
-        <v>44</v>
-      </c>
-      <c r="F23" s="1">
+      <c r="E23" s="1">
         <v>650</v>
       </c>
     </row>
@@ -2455,15 +2398,12 @@
         <v>83</v>
       </c>
       <c r="C24" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="D24" t="s">
         <v>52</v>
       </c>
-      <c r="E24" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="1">
+      <c r="E24" s="1">
         <v>3500</v>
       </c>
     </row>
@@ -2475,15 +2415,12 @@
         <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>220</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
         <v>55</v>
       </c>
-      <c r="E25" t="s">
-        <v>55</v>
-      </c>
-      <c r="F25" s="1">
+      <c r="E25" s="1">
         <v>16800</v>
       </c>
     </row>
@@ -2495,15 +2432,12 @@
         <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>219</v>
+        <v>97</v>
       </c>
       <c r="D26" t="s">
         <v>97</v>
       </c>
-      <c r="E26" t="s">
-        <v>97</v>
-      </c>
-      <c r="F26" s="1">
+      <c r="E26" s="1">
         <v>4000</v>
       </c>
     </row>
@@ -2514,17 +2448,17 @@
       <c r="B27" t="s">
         <v>90</v>
       </c>
-      <c r="C27" t="s">
-        <v>64</v>
+      <c r="C27" s="1" t="s">
+        <v>190</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="E27" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F27" s="1">
+      <c r="E27" s="1">
         <v>23100</v>
+      </c>
+      <c r="F27" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -2534,17 +2468,17 @@
       <c r="B28" t="s">
         <v>89</v>
       </c>
-      <c r="C28" t="s">
-        <v>64</v>
+      <c r="C28" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="E28" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="1">
+      <c r="E28" s="1">
         <v>27000</v>
+      </c>
+      <c r="F28" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
@@ -2554,16 +2488,13 @@
       <c r="B29" t="s">
         <v>91</v>
       </c>
-      <c r="C29" t="s">
-        <v>64</v>
+      <c r="C29" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F29" s="1">
+      <c r="E29" s="1">
         <v>17650</v>
       </c>
     </row>
@@ -2575,15 +2506,12 @@
         <v>93</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
         <v>67</v>
       </c>
-      <c r="E30" t="s">
-        <v>67</v>
-      </c>
-      <c r="F30" s="1">
+      <c r="E30" s="1">
         <v>90</v>
       </c>
     </row>
@@ -2595,15 +2523,12 @@
         <v>92</v>
       </c>
       <c r="C31" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
         <v>66</v>
       </c>
-      <c r="E31" t="s">
-        <v>66</v>
-      </c>
-      <c r="F31" s="1">
+      <c r="E31" s="1">
         <v>450</v>
       </c>
     </row>
@@ -2615,19 +2540,16 @@
         <v>94</v>
       </c>
       <c r="C32" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D32" t="s">
         <v>68</v>
       </c>
-      <c r="E32" t="s">
-        <v>68</v>
-      </c>
-      <c r="F32" s="1">
+      <c r="E32" s="1">
         <v>320</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>233</v>
       </c>
@@ -2635,19 +2557,16 @@
         <v>108</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
         <v>70</v>
       </c>
-      <c r="E33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F33" s="1">
+      <c r="E33" s="1">
         <v>1500</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>233</v>
       </c>
@@ -2655,23 +2574,13 @@
         <v>95</v>
       </c>
       <c r="C34" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
         <v>69</v>
       </c>
-      <c r="E34" t="s">
-        <v>69</v>
-      </c>
-      <c r="F34" s="1">
+      <c r="E34" s="1">
         <v>360</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D35"/>
-      <c r="F35" s="4">
-        <f>SUBTOTAL(109,BdBudgetPrevisionnel8[Provision])</f>
-        <v>175000</v>
       </c>
     </row>
   </sheetData>
@@ -2935,7 +2844,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
@@ -2956,7 +2865,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>210</v>
       </c>
@@ -3010,7 +2919,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>201</v>
       </c>
@@ -3037,7 +2946,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>210</v>
       </c>
@@ -3091,7 +3000,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>201</v>
       </c>
@@ -3118,7 +3027,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>210</v>
       </c>
@@ -3172,7 +3081,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>201</v>
       </c>
@@ -3199,7 +3108,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>210</v>
       </c>
@@ -3253,7 +3162,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -3274,7 +3183,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -3295,7 +3204,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -3322,7 +3231,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -3349,7 +3258,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>11</v>
       </c>
@@ -3376,7 +3285,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
@@ -3403,7 +3312,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
@@ -3431,7 +3340,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>26</v>
       </c>
@@ -3459,7 +3368,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
@@ -3483,7 +3392,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
@@ -3507,7 +3416,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>18</v>
       </c>
@@ -3535,7 +3444,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>18</v>
       </c>
@@ -3563,7 +3472,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>18</v>
       </c>
@@ -3591,7 +3500,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>24</v>
       </c>
@@ -3618,7 +3527,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>24</v>
       </c>
@@ -3645,7 +3554,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="87" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -3672,7 +3581,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>19</v>
       </c>
@@ -3699,7 +3608,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -3726,7 +3635,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>19</v>
       </c>
@@ -3753,7 +3662,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>19</v>
       </c>
@@ -3780,7 +3689,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>31</v>
       </c>
@@ -3801,7 +3710,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>18</v>
       </c>
@@ -3829,7 +3738,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>18</v>
       </c>
@@ -3857,7 +3766,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
@@ -3878,7 +3787,7 @@
         <v>3198.13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -3899,7 +3808,7 @@
         <v>3322.8</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>20</v>
       </c>
@@ -3920,7 +3829,7 @@
         <v>3138.27</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>19</v>
       </c>
@@ -3947,7 +3856,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>19</v>
       </c>
@@ -3974,7 +3883,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
@@ -4001,7 +3910,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>19</v>
       </c>
@@ -4028,7 +3937,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>125</v>
       </c>
@@ -4054,7 +3963,7 @@
       <c r="H44" s="5"/>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>125</v>
       </c>
@@ -4080,7 +3989,7 @@
       <c r="H45" s="5"/>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>125</v>
       </c>
@@ -4106,7 +4015,7 @@
       <c r="H46" s="5"/>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>125</v>
       </c>

</xml_diff>

<commit_message>
Protection en cas de temperature exterieur = residence
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="398" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD57C84B-8071-43E9-B1D5-8EE826D5B0A1}"/>
+  <xr:revisionPtr revIDLastSave="406" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBB2A207-7565-4E45-A442-BD117D0B57EF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -852,6 +852,9 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="50">
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1522,9 +1525,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1555,6 +1555,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="BdBudgetPrevisionnel8" displayName="BdBudgetPrevisionnel8" ref="A1:F34">
   <autoFilter ref="A1:F34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1563,7 +1567,7 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="0"/>
     <tableColumn id="5" xr3:uid="{2D489B7F-CE46-4597-8866-46E6A31D6BF8}" name="Top consommation chauffage"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1574,24 +1578,24 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}" name="BdCoproprietaires2" displayName="BdCoproprietaires2" ref="A1:P5" totalsRowShown="0">
   <autoFilter ref="A1:P5" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}"/>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="48"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="46">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="47">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="43"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="42"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="41"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="40"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="39"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="38"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="37"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="36"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="35"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="45"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="44"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="43"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="42"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="41"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="40"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="39"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="38"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="37"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="36"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1610,16 +1614,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="31"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="28">
       <calculatedColumnFormula>IF(BdCompetition9[[#This Row],[Taxes]]="TTC",BdCompetition9[[#This Row],[Cout]],BdCompetition9[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1632,16 +1636,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="20">
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="21">
       <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1658,7 +1662,7 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="19" totalsRowDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1671,23 +1675,23 @@
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="16">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="17">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="12"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="11"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="10"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="9"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="8"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="7"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="5"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="13"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="10"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
   </tableColumns>
@@ -1700,7 +1704,7 @@
   <autoFilter ref="A1:D9" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8584E7DE-3397-4839-B3F7-5BE29387C4A6}" name="Label des règles"/>
-    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{4C91DD63-5027-4E87-B95E-BCB801F28C1C}" name="Taxes"/>
     <tableColumn id="4" xr3:uid="{41CB6CC9-60A9-4712-874D-13D61D2EB5DE}" name="Total TTC">
       <calculatedColumnFormula>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</calculatedColumnFormula>
@@ -1715,7 +1719,7 @@
   <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2032,7 +2036,7 @@
         <v>101</v>
       </c>
       <c r="E2" s="1">
-        <v>1500</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -2049,7 +2053,7 @@
         <v>100</v>
       </c>
       <c r="E3" s="1">
-        <v>1500</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -2083,7 +2087,7 @@
         <v>102</v>
       </c>
       <c r="E5" s="1">
-        <v>2900</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -2117,7 +2121,7 @@
         <v>103</v>
       </c>
       <c r="E7" s="1">
-        <v>2900</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Les températures ne sont saisies qu'une fois au début, il faut maintenant refaire le calcul pour gérer la complémentarité des chaudières
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="406" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBB2A207-7565-4E45-A442-BD117D0B57EF}"/>
+  <xr:revisionPtr revIDLastSave="409" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD8E2B95-9F2F-4054-AC1A-699781D7F669}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="889" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="239">
   <si>
     <t>Montant</t>
   </si>
@@ -762,9 +762,6 @@
   </si>
   <si>
     <t>Top consommation chauffage</t>
-  </si>
-  <si>
-    <t>X</t>
   </si>
 </sst>
 </file>
@@ -852,9 +849,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="50">
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1525,6 +1519,9 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1567,7 +1564,7 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="48"/>
     <tableColumn id="5" xr3:uid="{2D489B7F-CE46-4597-8866-46E6A31D6BF8}" name="Top consommation chauffage"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1578,24 +1575,24 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}" name="BdCoproprietaires2" displayName="BdCoproprietaires2" ref="A1:P5" totalsRowShown="0">
   <autoFilter ref="A1:P5" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}"/>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="47"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="47">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="46">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="45"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="44"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="43"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="42"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="41"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="40"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="39"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="38"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="37"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="36"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="34"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="42"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="41"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="40"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="39"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="38"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="37"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="36"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="35"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1614,16 +1611,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="30"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="28">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="27">
       <calculatedColumnFormula>IF(BdCompetition9[[#This Row],[Taxes]]="TTC",BdCompetition9[[#This Row],[Cout]],BdCompetition9[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1636,16 +1633,16 @@
     <sortCondition ref="B1:B47"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{304F6CD1-2A85-4CA9-B82A-BF03CDAE07A4}" name="Type de prestation" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{068CBFB8-4A62-4CD4-BDAC-46EED59496BC}" name="Label de la prestation" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{2298CECF-E998-45F7-AABA-B59C715EC51B}" name="ID1" dataDxfId="23"/>
     <tableColumn id="3" xr3:uid="{5B85ADF0-B113-45E5-864A-388F8040031F}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="21">
+    <tableColumn id="4" xr3:uid="{037769D5-5B3A-4710-A4BD-50FC46B19887}" name="Cout" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{DDF49AF2-6301-4A34-B62A-4933E379FE46}" name="Taxes" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{D3462D22-93DD-4646-AC7F-1B3471D6826C}" name="Total TTC" dataDxfId="20">
       <calculatedColumnFormula>IF(BdCompetition[[#This Row],[Taxes]]="TTC",BdCompetition[[#This Row],[Cout]],BdCompetition[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{D6BDE268-55D6-4FDC-9C89-14F909955D72}" name="Description" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1662,7 +1659,7 @@
     <tableColumn id="5" xr3:uid="{F17C785C-9055-484D-A7EC-C3372D32A622}" name="Segment"/>
     <tableColumn id="7" xr3:uid="{3DB4DC80-D06E-4E70-BFE9-9BB75CB5FA62}" name="Classe de provision"/>
     <tableColumn id="2" xr3:uid="{3B6645ED-EDB5-4F76-9846-790ECF4F680D}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{EBBDC931-D4B2-4BFA-A08F-7BA2EEB44DAA}" name="Provision" totalsRowFunction="sum" dataDxfId="18" totalsRowDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1675,23 +1672,23 @@
     <tableColumn id="12" xr3:uid="{6157D014-929F-42D7-A4BC-12D951282608}" name="Batiment"/>
     <tableColumn id="4" xr3:uid="{81B9BF77-9818-477B-B3E8-1E987064DFDA}" name="Label de lot"/>
     <tableColumn id="1" xr3:uid="{B1F46291-565B-462F-9110-123FFF38DDEE}" name="Nom du coproprietaire"/>
-    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="17">
+    <tableColumn id="2" xr3:uid="{DE7A1664-88F0-47A5-B594-27860729EB7C}" name="Tantièmes copropriété" dataDxfId="16">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="13"/>
-    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="12"/>
-    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="10"/>
-    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="8"/>
-    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="7"/>
-    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="6"/>
-    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="4"/>
-    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{6082472F-2D58-4FBE-B207-F4E7921BE9CD}" name="Tantièmes ascenseur 1-1" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{A99085F3-5429-48BD-99D6-C368BEBDE1C5}" name="Tantièmes ascenseur 1-2" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{29D8D538-CA9C-4A95-992C-1A61F5728B38}" name="Tantièmes ascenseur 2" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{A8F24873-3570-4882-AE65-BFA97F5FA58C}" name="Tantièmes ascenseur 3" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{6A0D9C01-B4D3-4227-A105-5BE4105F433C}" name="Tantièmes chauffage" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{DB773FD9-45E5-4A17-9757-9A0D7F7768AA}" name="Tantièmes Batiment 1" dataDxfId="10"/>
+    <tableColumn id="16" xr3:uid="{2CD201B1-8753-466E-8776-252972944B3C}" name="Tantièmes Batiment 2" dataDxfId="9"/>
+    <tableColumn id="17" xr3:uid="{0EB76A3D-2FED-4CE0-9718-92F4FC209896}" name="Tantièmes Batiment 3" dataDxfId="8"/>
+    <tableColumn id="18" xr3:uid="{E820E31C-950D-4D14-8ABF-A71F86753025}" name="Tantièmes Hall 1-1" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{48F0D008-2EAA-4A4F-A6BA-4F8DF16617F8}" name="Tantièmes Hall 1-2" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{DD9B9883-76BB-4950-9FFB-0863C2F256EA}" name="Tantièmes Hall 2" dataDxfId="5"/>
+    <tableColumn id="21" xr3:uid="{BF704940-4EA2-48AF-8BBA-B1F4C695A5E2}" name="Tantièmes Logement/Stationnements" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{23C5575F-C8F7-420A-A8AC-4CD0404C3FB6}" name="Stationnement" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{4AF86A31-E98F-489D-ABE5-CCD678E7BE8D}" name="Numéro de lot" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{71861424-FDE4-4C97-8393-5794B9911F90}" name="Lot Nexity"/>
     <tableColumn id="5" xr3:uid="{99825B0E-48FC-48C3-B40C-A8763FC406C7}" name="Etage"/>
   </tableColumns>
@@ -1704,7 +1701,7 @@
   <autoFilter ref="A1:D9" xr:uid="{594FE941-6967-448D-B161-1A22202460B2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8584E7DE-3397-4839-B3F7-5BE29387C4A6}" name="Label des règles"/>
-    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2DAB5E09-C6DA-4A52-9D36-12A8D2B9BE1E}" name="Limite" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{4C91DD63-5027-4E87-B95E-BCB801F28C1C}" name="Taxes"/>
     <tableColumn id="4" xr3:uid="{41CB6CC9-60A9-4712-874D-13D61D2EB5DE}" name="Total TTC">
       <calculatedColumnFormula>IF(BdRegles[[#This Row],[Taxes]]="HT",BdRegles[[#This Row],[Limite]]*1.2,BdRegles[[#This Row],[Limite]])</calculatedColumnFormula>
@@ -1719,7 +1716,7 @@
   <autoFilter ref="A1:B2" xr:uid="{B8BAE385-571F-4715-A042-0AD7A1FDF085}"/>
   <tableColumns count="2">
     <tableColumn id="2" xr3:uid="{75AB35E7-AA7F-46C7-B30C-DC2E9C862FFF}" name="Label du revenu"/>
-    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4F014B57-0040-4CC7-87A1-9B988F634586}" name="Montant" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1998,7 +1995,7 @@
     <col min="2" max="2" width="15.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="42.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2461,8 +2458,8 @@
       <c r="E27" s="1">
         <v>23100</v>
       </c>
-      <c r="F27" t="s">
-        <v>239</v>
+      <c r="F27">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -2481,8 +2478,8 @@
       <c r="E28" s="1">
         <v>27000</v>
       </c>
-      <c r="F28" t="s">
-        <v>239</v>
+      <c r="F28">
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Calculs chauffage central fait mais vérifier résultats
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Victor Diné\OneDrive\Documents\Mon Patrimoine\Projet Immobilier\2023 Terrasses de Galieni\09 - Copropriété\Site de calcul des charges de copropriété\streamlit-copro-charges\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="493" documentId="13_ncr:1_{BC6B5EAF-A22B-4219-B771-90D3DDB91BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{294AA836-5EE7-44F2-8CB2-D18602EDAD37}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="217">
   <si>
     <t>Taxes</t>
   </si>
@@ -455,9 +455,6 @@
     <t>Estimation faite car absent du contrat; 1ère année offerte</t>
   </si>
   <si>
-    <t>Eontrat  P2, engagement sur 3 ans</t>
-  </si>
-  <si>
     <t>Option traitement adoucissant eau avec engagement sur 3 ans</t>
   </si>
   <si>
@@ -690,6 +687,12 @@
   </si>
   <si>
     <t>Terrasses de Gallieni</t>
+  </si>
+  <si>
+    <t>Ordre d'utilisation</t>
+  </si>
+  <si>
+    <t>Contrat  P2, engagement sur 3 ans</t>
   </si>
 </sst>
 </file>
@@ -1140,10 +1143,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:E34">
   <autoFilter ref="A1:E34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1221,13 +1220,14 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:E3" totalsRowShown="0">
+  <autoFilter ref="A1:E3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
     <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="24" dataCellStyle="Currency"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kWh"/>
+    <tableColumn id="5" xr3:uid="{ED1B8FB3-6899-430D-BDC7-A9BDBA679526}" name="Ordre d'utilisation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1500,25 +1500,25 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D1" t="s">
         <v>96</v>
@@ -1527,15 +1527,15 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
         <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D2" t="s">
         <v>84</v>
@@ -1544,15 +1544,15 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B3" t="s">
         <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D3" t="s">
         <v>83</v>
@@ -1561,32 +1561,32 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E4" s="1">
         <v>2000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
         <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D5" t="s">
         <v>85</v>
@@ -1595,32 +1595,32 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6" s="1">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B7" t="s">
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D7" t="s">
         <v>86</v>
@@ -1629,26 +1629,26 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E8" s="1">
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B9" t="s">
         <v>68</v>
@@ -1663,9 +1663,9 @@
         <v>750</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B10" t="s">
         <v>67</v>
@@ -1680,9 +1680,9 @@
         <v>6200</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s">
         <v>64</v>
@@ -1697,9 +1697,9 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B12" t="s">
         <v>63</v>
@@ -1714,9 +1714,9 @@
         <v>900</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B13" t="s">
         <v>62</v>
@@ -1731,9 +1731,9 @@
         <v>920</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B14" t="s">
         <v>55</v>
@@ -1748,9 +1748,9 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
         <v>56</v>
@@ -1765,9 +1765,9 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B16" t="s">
         <v>65</v>
@@ -1782,9 +1782,9 @@
         <v>580</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B17" t="s">
         <v>70</v>
@@ -1799,9 +1799,9 @@
         <v>570</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B18" t="s">
         <v>71</v>
@@ -1816,9 +1816,9 @@
         <v>850</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B19" t="s">
         <v>60</v>
@@ -1833,9 +1833,9 @@
         <v>240</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B20" t="s">
         <v>59</v>
@@ -1850,9 +1850,9 @@
         <v>220</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B21" t="s">
         <v>57</v>
@@ -1867,9 +1867,9 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B22" t="s">
         <v>61</v>
@@ -1882,9 +1882,9 @@
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B23" t="s">
         <v>58</v>
@@ -1899,9 +1899,9 @@
         <v>650</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s">
         <v>66</v>
@@ -1916,9 +1916,9 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B25" t="s">
         <v>69</v>
@@ -1933,9 +1933,9 @@
         <v>16800</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B26" t="s">
         <v>79</v>
@@ -1950,15 +1950,15 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B27" t="s">
         <v>73</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>48</v>
@@ -1967,15 +1967,15 @@
         <v>23100</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B28" t="s">
         <v>72</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>47</v>
@@ -1984,9 +1984,9 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B29" t="s">
         <v>74</v>
@@ -2001,9 +2001,9 @@
         <v>17650</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B30" t="s">
         <v>76</v>
@@ -2018,9 +2018,9 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B31" t="s">
         <v>75</v>
@@ -2035,9 +2035,9 @@
         <v>450</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
         <v>77</v>
@@ -2052,9 +2052,9 @@
         <v>320</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B33" t="s">
         <v>91</v>
@@ -2069,9 +2069,9 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B34" t="s">
         <v>78</v>
@@ -2100,77 +2100,77 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="21.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C1" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="H1" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="G1" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="O1" s="9" t="s">
-        <v>159</v>
-      </c>
       <c r="P1" s="9" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>225</v>
       </c>
       <c r="B2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C2" s="9">
         <v>217</v>
@@ -2199,12 +2199,12 @@
       </c>
       <c r="P2" s="9"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>308</v>
       </c>
       <c r="B3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C3" s="9">
         <v>82</v>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="P3" s="9"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>113</v>
       </c>
       <c r="B4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C4" s="9">
         <v>86</v>
@@ -2265,12 +2265,12 @@
       </c>
       <c r="P4" s="9"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>462</v>
       </c>
       <c r="B5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C5" s="9">
         <v>7</v>
@@ -2309,19 +2309,19 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:I47"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.1796875" customWidth="1"/>
-    <col min="2" max="2" width="66.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="159.7265625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="48.140625" customWidth="1"/>
+    <col min="2" max="2" width="66.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="159.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>106</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>95</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D1" t="s">
         <v>94</v>
@@ -2344,10 +2344,10 @@
         <v>3</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>23</v>
       </c>
@@ -2368,18 +2368,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E3" s="5">
         <v>0</v>
@@ -2392,21 +2392,21 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E4" s="5">
         <v>10000</v>
@@ -2419,21 +2419,21 @@
         <v>10000</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E5" s="5">
         <v>16000</v>
@@ -2446,21 +2446,21 @@
         <v>16000</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E6" s="5">
         <v>1940</v>
@@ -2473,21 +2473,21 @@
         <v>1940</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E7" s="5">
         <v>18000</v>
@@ -2500,21 +2500,21 @@
         <v>18000</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E8" s="5">
         <v>24000</v>
@@ -2527,21 +2527,21 @@
         <v>24000</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E9" s="5">
         <v>5710</v>
@@ -2554,21 +2554,21 @@
         <v>5710</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E10" s="5">
         <v>20000</v>
@@ -2581,21 +2581,21 @@
         <v>20000</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E11" s="5">
         <v>37000</v>
@@ -2608,21 +2608,21 @@
         <v>37000</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E12" s="5">
         <v>10770</v>
@@ -2635,21 +2635,21 @@
         <v>10770</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E13" s="5">
         <v>25000</v>
@@ -2662,10 +2662,10 @@
         <v>25000</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>8</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2840,10 +2840,10 @@
         <v>16750</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -2868,10 +2868,10 @@
         <v>887</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>12</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>12</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>12</v>
       </c>
@@ -3003,7 +3003,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>18</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>18</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
@@ -3084,12 +3084,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C30" t="s">
         <v>87</v>
@@ -3111,12 +3111,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C31" t="s">
         <v>88</v>
@@ -3138,12 +3138,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C32" t="s">
         <v>89</v>
@@ -3165,12 +3165,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C33" t="s">
         <v>90</v>
@@ -3192,7 +3192,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>25</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>12</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>12</v>
       </c>
@@ -3269,7 +3269,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>3198.13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>14</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>3322.8</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>14</v>
       </c>
@@ -3332,12 +3332,12 @@
         <v>3138.27</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C40" t="s">
         <v>87</v>
@@ -3359,12 +3359,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C41" t="s">
         <v>88</v>
@@ -3386,12 +3386,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C42" t="s">
         <v>89</v>
@@ -3413,12 +3413,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C43" t="s">
         <v>90</v>
@@ -3440,18 +3440,18 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>100</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D44" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E44" s="6">
         <v>10000</v>
@@ -3466,18 +3466,18 @@
       <c r="H44" s="4"/>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E45" s="6">
         <v>12500</v>
@@ -3492,18 +3492,18 @@
       <c r="H45" s="4"/>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>100</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D46" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E46" s="6">
         <v>15000</v>
@@ -3518,7 +3518,7 @@
       <c r="H46" s="4"/>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>100</v>
       </c>
@@ -3565,30 +3565,31 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1796875" customWidth="1"/>
-    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>214</v>
-      </c>
-      <c r="B1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>215</v>
       </c>
       <c r="B2">
         <v>10007</v>
@@ -3613,32 +3614,36 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.54296875" customWidth="1"/>
-    <col min="3" max="3" width="21.26953125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.6328125" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" t="s">
         <v>207</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" t="s">
         <v>209</v>
       </c>
-      <c r="D1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>72</v>
@@ -3650,10 +3655,13 @@
       <c r="D2">
         <v>150</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B3" t="s">
         <v>73</v>
@@ -3663,6 +3671,9 @@
       </c>
       <c r="D3">
         <v>225</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction bug chauffage central
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Victor Diné\OneDrive\Documents\Mon Patrimoine\Projet Immobilier\2023 Terrasses de Galieni\09 - Copropriété\Site de calcul des charges de copropriété\streamlit-copro-charges\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{292F8C4A-B358-465D-91BA-601DADA9744A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="218">
   <si>
     <t>Taxes</t>
   </si>
@@ -671,9 +671,6 @@
     <t>Prix unitaire du kWh</t>
   </si>
   <si>
-    <t>Production maximum en kWh</t>
-  </si>
-  <si>
     <t>Atlantic Varmax 2 225</t>
   </si>
   <si>
@@ -693,6 +690,12 @@
   </si>
   <si>
     <t>Contrat  P2, engagement sur 3 ans</t>
+  </si>
+  <si>
+    <t>Production maximum en kW</t>
+  </si>
+  <si>
+    <t>Option adoucissant eau CRAM</t>
   </si>
 </sst>
 </file>
@@ -1143,6 +1146,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:E34">
   <autoFilter ref="A1:E34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1226,7 +1233,7 @@
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
     <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="24" dataCellStyle="Currency"/>
-    <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kWh"/>
+    <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="5" xr3:uid="{ED1B8FB3-6899-430D-BDC7-A9BDBA679526}" name="Ordre d'utilisation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2840,7 +2847,7 @@
         <v>16750</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2848,7 +2855,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>128</v>
+        <v>217</v>
       </c>
       <c r="C21" t="s">
         <v>74</v>
@@ -3575,13 +3582,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B1" t="s">
         <v>204</v>
       </c>
       <c r="C1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D1" t="s">
         <v>205</v>
@@ -3589,7 +3596,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2">
         <v>10007</v>
@@ -3620,7 +3627,7 @@
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3635,15 +3642,15 @@
         <v>208</v>
       </c>
       <c r="D1" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="E1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>72</v>
@@ -3661,7 +3668,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B3" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
Ajout de description aux provisions, mettre les prestation élus en défaut. Ajout de barre de navigation
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{292F8C4A-B358-465D-91BA-601DADA9744A}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65E87D2B-FC20-4094-AC79-916EE09F4D58}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="234">
   <si>
     <t>Taxes</t>
   </si>
@@ -674,9 +674,6 @@
     <t>Atlantic Varmax 2 225</t>
   </si>
   <si>
-    <t>Herz Firematic 150</t>
-  </si>
-  <si>
     <t>Volume à chauffer en m3</t>
   </si>
   <si>
@@ -696,6 +693,68 @@
   </si>
   <si>
     <t>Option adoucissant eau CRAM</t>
+  </si>
+  <si>
+    <t>Prix du granulé: Gruchy = 310€/t, CRAM = 392€/t et Prochalor 500€/t</t>
+  </si>
+  <si>
+    <t>Herz Firematic 20-60</t>
+  </si>
+  <si>
+    <t>Chaudière d'appoint au gaz</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Entretien porte de parking Eurosofia</t>
+  </si>
+  <si>
+    <t>Eurosofia</t>
+  </si>
+  <si>
+    <t>Rajouté</t>
+  </si>
+  <si>
+    <t>Prestation choisie actuellement</t>
+  </si>
+  <si>
+    <t>Un contrat « ferme-porte » (souvent appelé contrat fermé, par opposition à un contrat « ouvert ») est une modalité de contrat de maintenance et d'entretien, généralement souscrit par le syndicat des copropriétaires pour certains équipements communs (le plus souvent la porte automatique de garage / parking, le portail, ou parfois l'ascenseur).</t>
+  </si>
+  <si>
+    <t>C'est un pot commun d'heures ou d'interventions attribué à un sous-traitant (ou au gardien/maintenance) pour effectuer de petits travaux courants sans avoir à repasser par une demande de devis, un vote du conseil syndical ou un ordre de service formel du syndic à chaque micro-problème.
+Le prestataire dispose d'une marge de manœuvre (le « bac à sable ») pour agir en autonomie ou sur simple signalement dans la limite du forfait.</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance du désenfumage est une prestation souscrite par le syndicat des copropriétaires pour assurer le bon fonctionnement, la vérification périodique et l'entretien des installations de désenfumage de l'immeuble (les exutoires de fumée en cage d'escalier, les volets, les gaines et les centrales de commande).
+C'est un contrat de maintenance obligatoire et réglementaire, essentiel pour la sécurité incendie de la copropriété.</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance pour pompe de relevage est une convention souscrite par la copropriété auprès d'un prestataire spécialisé (assainissement, plomberie industrielle) pour assurer l'entretien, le contrôle et le dépannage de la ou des pompes situées dans les sous-sols de l'immeuble.
+C'est un contrat critique pour la salubrité de l'immeuble et la prévention des inondations, en particulier au niveau des sous-sols et des parkings.</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance de la ventilation de parking (aussi appelée désenfumage mécanique ou extraction du parking) est une prestation souscrite par le syndicat des copropriétaires pour assurer l'entretien et le bon fonctionnement des équipements d'aération et d'extraction d'air dans les sous-sols et garages de l'immeuble.
+C'est un contrat de sécurité obligatoire et réglementaire dès lors que le parking répond à certaines caractéristiques (nombre de niveaux ou de places).</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance des colonnes sèches est une prestation obligatoire souscrite par le syndicat des copropriétaires pour garantir le bon état de fonctionnement et la résistance sous pression des tuyauteries d'incendie installées dans l'immeuble.
+🚒 À quoi sert une colonne sèche ?
+Une colonne sèche est un tuyau vide fixé verticalement dans la cage d'escalier (ou une gaine technique) reliant le rez-de-chaussée (ou l'extérieur) aux différents étages de l'immeuble.
+En temps normal : La conduite est vide d'eau (d'où le terme « sèche »).
+En cas d'incendie : Les pompiers raccordent leur camion-citerne à l'orifice d'alimentation situé au bas de l'immeuble pour y injecter de l'eau sous forte pression. Ils n'ont plus qu'à monter aux étages concernés et brancher leurs lances directement sur la prise d'étage.
+L'objectif principal : Éviter aux pompiers de devoir dérouler des centaines de mètres de tuyaux dans les escaliers, ce qui fait gagner des minutes précieuses.</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance du désenfumage en circulation est la prestation souscrite par la copropriété pour contrôler et entretenir les installations d'évacuation de fumée spécifiques aux espaces communs horizontaux de l'immeuble (couloirs, coursives, sas d'accès).
+Il s'agit d'une déclinaison précise du contrat de sécurité incendie global, axée sur les zones de passage qui relient les appartements à la cage d'escalier ou aux sorties.</t>
+  </si>
+  <si>
+    <t>Un contrat de maintenance des blocs de secours (souvent abrégé BAES pour Blocs Autonomes d'Éclairage de Sécurité) est un contrat souscrit par la copropriété pour assurer le bon fonctionnement, la vérification réglementaire et le remplacement des boîtiers lumineux d'urgence installés dans les parties communes.
+Ce sont les petits boîtiers rectangulaires blancs (souvent dotés d'un pictogramme vert avec un bonhomme qui court) situés au-dessus des portes de sortie, dans les cages d'escalier, les couloirs et les sous-sols/parkings.</t>
+  </si>
+  <si>
+    <t>Description longue</t>
   </si>
 </sst>
 </file>
@@ -787,7 +846,31 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="27">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1115,24 +1198,6 @@
         <scheme val="minor"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1151,14 +1216,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:E34">
-  <autoFilter ref="A1:E34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:F34">
+  <autoFilter ref="A1:F34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F34">
+    <sortCondition descending="1" ref="E1:E34"/>
+  </sortState>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3B91602D-BA59-47C1-AD19-EAA938B961C7}" name="ID tantiemes"/>
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1168,46 +1237,47 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}" name="Lots" displayName="Lots" ref="A1:P5" totalsRowShown="0">
   <autoFilter ref="A1:P5" xr:uid="{74E83642-0ED6-4017-A369-70F6DD3FC748}"/>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="24"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="20">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="23">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="18"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="16"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="15"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="14"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="11"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="9"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="19"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="18"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="17"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="16"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="15"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="13"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:H47" totalsRowShown="0">
-  <autoFilter ref="A1:H47" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H47">
-    <sortCondition ref="B1:B47"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I48" totalsRowShown="0">
+  <autoFilter ref="A1:I48" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H48">
+    <sortCondition ref="B1:B48"/>
   </sortState>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="4"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="4">
       <calculatedColumnFormula>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1227,14 +1297,15 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:E3" totalsRowShown="0">
-  <autoFilter ref="A1:E3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:F3" totalsRowShown="0">
+  <autoFilter ref="A1:F3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
-    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="24" dataCellStyle="Currency"/>
+    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="26" dataCellStyle="Currency"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="5" xr3:uid="{ED1B8FB3-6899-430D-BDC7-A9BDBA679526}" name="Ordre d'utilisation"/>
+    <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1506,7 +1577,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
@@ -1514,10 +1585,10 @@
     <col min="3" max="3" width="42.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="42.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="147" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>203</v>
       </c>
@@ -1533,565 +1604,617 @@
       <c r="E1" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>164</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="E2" s="1">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>35000</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D3" t="s">
-        <v>83</v>
+        <v>72</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="E3" s="1">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>27000</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D4" t="s">
-        <v>168</v>
+        <v>73</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="E4" s="1">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>23100</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>166</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="E5" s="1">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18000</v>
+      </c>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C6" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" t="s">
-        <v>169</v>
+        <v>74</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E6" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17650</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>187</v>
+        <v>147</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>167</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="E7" s="1">
-        <v>2700</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16800</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>163</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>170</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>170</v>
+        <v>42</v>
       </c>
       <c r="E8" s="1">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>6200</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="E9" s="1">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4000</v>
+      </c>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="1">
-        <v>6200</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>3500</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>166</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>85</v>
       </c>
       <c r="E11" s="1">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>3000</v>
+      </c>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>164</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="E12" s="1">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2900</v>
+      </c>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="E13" s="1">
-        <v>920</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2900</v>
+      </c>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="E14" s="1">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2700</v>
+      </c>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>161</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>168</v>
       </c>
       <c r="E15" s="1">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2000</v>
+      </c>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>147</v>
       </c>
       <c r="B16" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="D16" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E16" s="1">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1500</v>
+      </c>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="E17" s="1">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1500</v>
+      </c>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>147</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E18" s="1">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1050</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>162</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>169</v>
       </c>
       <c r="D19" t="s">
-        <v>35</v>
+        <v>169</v>
       </c>
       <c r="E19" s="1">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1000</v>
+      </c>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>163</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
+        <v>170</v>
       </c>
       <c r="D20" t="s">
-        <v>34</v>
+        <v>170</v>
       </c>
       <c r="E20" s="1">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1000</v>
+      </c>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>147</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E21" s="1">
-        <v>18000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+        <v>920</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>147</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
-      </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="E22" s="1">
+        <v>900</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>147</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="E23" s="1">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <v>850</v>
+      </c>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D24" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E24" s="1">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <v>750</v>
+      </c>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>147</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D25" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="E25" s="1">
-        <v>16800</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="D26" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E26" s="1">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>580</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>48</v>
+        <v>70</v>
+      </c>
+      <c r="C27" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" t="s">
+        <v>45</v>
       </c>
       <c r="E27" s="1">
-        <v>23100</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>570</v>
+      </c>
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>47</v>
+        <v>75</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" t="s">
+        <v>50</v>
       </c>
       <c r="E28" s="1">
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>49</v>
+        <v>78</v>
+      </c>
+      <c r="C29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D29" t="s">
+        <v>53</v>
       </c>
       <c r="E29" s="1">
-        <v>17650</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>199</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E30" s="1">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>320</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>199</v>
+        <v>147</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="D31" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E31" s="1">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>147</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="D32" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E32" s="1">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>199</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E33" s="1">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>199</v>
+        <v>147</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="D34" t="s">
-        <v>53</v>
-      </c>
-      <c r="E34" s="1">
-        <v>360</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E34" s="1"/>
+      <c r="F34" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2315,7 +2438,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.140625" customWidth="1"/>
@@ -2325,10 +2448,11 @@
     <col min="5" max="5" width="11.85546875" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="159.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="71.5703125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="48.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>106</v>
       </c>
@@ -2353,8 +2477,11 @@
       <c r="H1" s="10" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>23</v>
       </c>
@@ -2375,7 +2502,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>180</v>
       </c>
@@ -2402,7 +2529,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>179</v>
       </c>
@@ -2429,7 +2556,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>171</v>
       </c>
@@ -2456,7 +2583,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>180</v>
       </c>
@@ -2483,7 +2610,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>179</v>
       </c>
@@ -2510,7 +2637,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>171</v>
       </c>
@@ -2537,7 +2664,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>180</v>
       </c>
@@ -2564,7 +2691,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>179</v>
       </c>
@@ -2591,7 +2718,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>171</v>
       </c>
@@ -2618,7 +2745,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>180</v>
       </c>
@@ -2645,7 +2772,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>179</v>
       </c>
@@ -2672,7 +2799,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
@@ -2693,7 +2820,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
@@ -2714,7 +2841,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>28</v>
       </c>
@@ -2741,7 +2868,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>8</v>
       </c>
@@ -2767,8 +2894,11 @@
       <c r="H17" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
@@ -2794,8 +2924,11 @@
       <c r="H18" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -2822,7 +2955,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
@@ -2847,15 +2980,15 @@
         <v>16750</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C21" t="s">
         <v>74</v>
@@ -2878,7 +3011,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -2902,7 +3035,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>20</v>
       </c>
@@ -2926,7 +3059,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>12</v>
       </c>
@@ -2954,7 +3087,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>12</v>
       </c>
@@ -2982,7 +3115,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>12</v>
       </c>
@@ -3009,8 +3142,11 @@
       <c r="H26" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I26" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>18</v>
       </c>
@@ -3037,7 +3173,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>18</v>
       </c>
@@ -3064,7 +3200,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="225" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>18</v>
       </c>
@@ -3091,42 +3227,45 @@
         <v>133</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>139</v>
+        <v>221</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>222</v>
       </c>
       <c r="E30" s="5">
-        <v>2400</v>
+        <v>434.5</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2880</v>
+        <v>434.5</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D31" t="s">
         <v>81</v>
@@ -3144,32 +3283,38 @@
       <c r="H31" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I31" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D32" t="s">
         <v>81</v>
       </c>
       <c r="E32" s="5">
-        <v>2450</v>
+        <v>2400</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>1</v>
       </c>
       <c r="G32" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2940</v>
+        <v>2880</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>135</v>
+      </c>
+      <c r="I32" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -3177,75 +3322,80 @@
         <v>13</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D33" t="s">
         <v>81</v>
       </c>
       <c r="E33" s="5">
-        <v>2200</v>
+        <v>2450</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>1</v>
       </c>
       <c r="G33" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2640</v>
+        <v>2940</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="I33" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>25</v>
+        <v>146</v>
+      </c>
+      <c r="C34" t="s">
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="E34" s="5">
-        <v>160</v>
+        <v>2200</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>160</v>
+        <v>2640</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I34" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="D35" t="s">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="E35" s="5">
-        <f>2400*12</f>
-        <v>28800</v>
+        <v>160</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>2</v>
       </c>
       <c r="G35" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>28800</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>109</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -3253,7 +3403,7 @@
         <v>12</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C36" t="s">
         <v>57</v>
@@ -3262,39 +3412,46 @@
         <v>110</v>
       </c>
       <c r="E36" s="5">
+        <f>2400*12</f>
+        <v>28800</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G36" s="5">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>28800</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C37" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" t="s">
+        <v>110</v>
+      </c>
+      <c r="E37" s="5">
         <f>1320*12</f>
         <v>15840</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G36" s="5">
+      <c r="F37" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G37" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
         <v>15840</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D37" t="s">
-        <v>17</v>
-      </c>
-      <c r="E37" s="5">
-        <v>3198.13</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G37" s="5">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3198.13</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -3302,20 +3459,20 @@
         <v>14</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D38" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E38" s="5">
-        <v>3322.8</v>
+        <v>3198.13</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>2</v>
       </c>
       <c r="G38" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3322.8</v>
+        <v>3198.13</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -3323,47 +3480,41 @@
         <v>14</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D39" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E39" s="5">
-        <v>3138.27</v>
+        <v>3322.8</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>2</v>
       </c>
       <c r="G39" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3138.27</v>
+        <v>3322.8</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C40" t="s">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="D40" t="s">
-        <v>81</v>
+        <v>15</v>
       </c>
       <c r="E40" s="5">
-        <v>240</v>
+        <v>3138.27</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>288</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>135</v>
+        <v>3138.27</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -3371,10 +3522,10 @@
         <v>13</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C41" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D41" t="s">
         <v>81</v>
@@ -3398,10 +3549,10 @@
         <v>13</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D42" t="s">
         <v>81</v>
@@ -3425,10 +3576,10 @@
         <v>13</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D43" t="s">
         <v>81</v>
@@ -3449,36 +3600,37 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>69</v>
+        <v>145</v>
+      </c>
+      <c r="C44" t="s">
+        <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>188</v>
-      </c>
-      <c r="E44" s="6">
-        <v>10000</v>
-      </c>
-      <c r="F44" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G44" s="6">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>10000</v>
-      </c>
-      <c r="H44" s="4"/>
-      <c r="I44" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="E44" s="5">
+        <v>240</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G44" s="5">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>288</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>69</v>
@@ -3487,14 +3639,14 @@
         <v>188</v>
       </c>
       <c r="E45" s="6">
-        <v>12500</v>
+        <v>10000</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>2</v>
       </c>
       <c r="G45" s="6">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>12500</v>
+        <v>10000</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="2"/>
@@ -3504,7 +3656,7 @@
         <v>100</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>69</v>
@@ -3513,14 +3665,14 @@
         <v>188</v>
       </c>
       <c r="E46" s="6">
-        <v>15000</v>
+        <v>12500</v>
       </c>
       <c r="F46" s="8" t="s">
         <v>2</v>
       </c>
       <c r="G46" s="6">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>15000</v>
+        <v>12500</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="2"/>
@@ -3530,32 +3682,60 @@
         <v>100</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>100</v>
+        <v>190</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D47" t="s">
+        <v>188</v>
+      </c>
+      <c r="E47" s="6">
+        <v>15000</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G47" s="6">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>15000</v>
+      </c>
+      <c r="H47" s="4"/>
+      <c r="I47" s="2"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D48" t="s">
         <v>27</v>
       </c>
-      <c r="E47" s="6">
+      <c r="E48" s="6">
         <v>16800</v>
       </c>
-      <c r="F47" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G47" s="6">
+      <c r="F48" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G48" s="6">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
         <v>16800</v>
       </c>
-      <c r="H47" s="4" t="s">
+      <c r="H48" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="I47" s="2"/>
+      <c r="I48" s="2" t="s">
+        <v>220</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C47" xr:uid="{10A37FDE-E67C-425C-BC79-E21761381591}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C48" xr:uid="{10A37FDE-E67C-425C-BC79-E21761381591}">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -3582,13 +3762,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B1" t="s">
         <v>204</v>
       </c>
       <c r="C1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D1" t="s">
         <v>205</v>
@@ -3596,7 +3776,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B2">
         <v>10007</v>
@@ -3621,17 +3801,18 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="61.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>206</v>
       </c>
@@ -3642,31 +3823,37 @@
         <v>208</v>
       </c>
       <c r="D1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+      <c r="F1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>72</v>
       </c>
       <c r="C2" s="1">
-        <f>392/4600</f>
-        <v>8.5217391304347828E-2</v>
+        <f>310*1.2/4600</f>
+        <v>8.0869565217391304E-2</v>
       </c>
       <c r="D2">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>209</v>
       </c>
@@ -3681,6 +3868,9 @@
       </c>
       <c r="E3">
         <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Suppression de la classe lot réussie, simplifications en cours, je vais essayer d'intégrer le calcul de la consommation en eau
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="690" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8042C2AA-65EE-4305-8FA3-CD53475E7F32}"/>
+  <xr:revisionPtr revIDLastSave="708" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A140CCE-984B-4FAC-939A-1C0CB3B44D57}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="251">
   <si>
     <t>Taxes</t>
   </si>
@@ -687,9 +687,6 @@
   </si>
   <si>
     <t>Prix du granulé: Gruchy = 310€/t, CRAM = 392€/t et Prochalor 500€/t</t>
-  </si>
-  <si>
-    <t>Herz Firematic 20-60</t>
   </si>
   <si>
     <t>Chaudière d'appoint au gaz</t>
@@ -785,6 +782,31 @@
   </si>
   <si>
     <t>Lot 113 - T2 45m2 3ème étage Batiment 1.1 exposé nord/est</t>
+  </si>
+  <si>
+    <t>Herz Firematic 130</t>
+  </si>
+  <si>
+    <t>De 310€/t pour Gruchy à 500€/t pour Prochalor</t>
+  </si>
+  <si>
+    <t>Contrat associé à la porte principale du parking souterrain</t>
+  </si>
+  <si>
+    <t>Assistance juridique à la copropriété</t>
+  </si>
+  <si>
+    <t>Electricité du bâtiment 1: éclairages couloirs, éclairages hall, interphones. Relié aux panneaux solaires, avec revente du surplus d'électricité.</t>
+  </si>
+  <si>
+    <t>Electricité du bâtiment 2: éclairages couloirs, éclairages hall, interphones. Relié aux panneaux solaires, avec revente du surplus d'électricité.</t>
+  </si>
+  <si>
+    <t>Electricité du bâtiment 3: éclairages couloirs, éclairages hall, interphones. Relié aux panneaux solaires, avec revente du surplus d'électricité.</t>
+  </si>
+  <si>
+    <t>La facturation par Est Ensemble est progressive, gratuit jusqu'à 10m3, puis de 10 à 28 m³ = 1,1988 € HT / m³, de 28 à 86 m³ = 1,3320 € HT / m³, de 86 à 101 m³ = 1,3720 € HT / m³, de 101 à 131 m³ = 1,4200 € HT / m³, de 131 à 140 m³ = 1,4919 € HT / m³ et Plus de 140 m³ = 1,5366 € HT / m³
+On rajoute la redevance (3,3€/m3) et la TVA (8%)</t>
   </si>
 </sst>
 </file>
@@ -1240,6 +1262,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:F34">
   <autoFilter ref="A1:F34" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1632,10 +1658,10 @@
         <v>97</v>
       </c>
       <c r="F1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>147</v>
       </c>
@@ -1651,7 +1677,9 @@
       <c r="E2" s="1">
         <v>35000</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1669,7 +1697,9 @@
       <c r="E3" s="1">
         <v>27000</v>
       </c>
-      <c r="F3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -1885,7 +1915,9 @@
       <c r="E15" s="1">
         <v>2000</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1940,7 +1972,7 @@
         <v>1050</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1959,7 +1991,9 @@
       <c r="E19" s="1">
         <v>1000</v>
       </c>
-      <c r="F19" s="2"/>
+      <c r="F19" s="2" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1977,7 +2011,9 @@
       <c r="E20" s="1">
         <v>1000</v>
       </c>
-      <c r="F20" s="2"/>
+      <c r="F20" s="2" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1996,7 +2032,7 @@
         <v>920</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -2016,7 +2052,7 @@
         <v>900</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2053,7 +2089,9 @@
       <c r="E24" s="1">
         <v>750</v>
       </c>
-      <c r="F24" s="2"/>
+      <c r="F24" s="2" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -2090,7 +2128,7 @@
         <v>580</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2127,7 +2165,9 @@
       <c r="E28" s="1">
         <v>450</v>
       </c>
-      <c r="F28" s="2"/>
+      <c r="F28" s="2" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -2146,7 +2186,7 @@
         <v>360</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2166,7 +2206,7 @@
         <v>320</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2186,7 +2226,7 @@
         <v>240</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2224,7 +2264,7 @@
         <v>90</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2327,7 +2367,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C2">
         <v>462</v>
@@ -2341,7 +2381,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C3">
         <v>119</v>
@@ -2367,7 +2407,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C4">
         <v>83</v>
@@ -2393,7 +2433,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5">
         <v>130</v>
@@ -2419,7 +2459,7 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -2445,7 +2485,7 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C7">
         <v>122</v>
@@ -2471,7 +2511,7 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C8">
         <v>55</v>
@@ -2497,7 +2537,7 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C9">
         <v>96</v>
@@ -2523,7 +2563,7 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C10">
         <v>123</v>
@@ -2549,7 +2589,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C11">
         <v>129</v>
@@ -2575,7 +2615,7 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C12">
         <v>58</v>
@@ -2601,7 +2641,7 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C13">
         <v>91</v>
@@ -2627,7 +2667,7 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C14" s="8">
         <v>86</v>
@@ -6493,7 +6533,7 @@
         <v>138</v>
       </c>
       <c r="I1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -6910,7 +6950,7 @@
         <v>93</v>
       </c>
       <c r="I17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -6940,7 +6980,7 @@
         <v>102</v>
       </c>
       <c r="I18" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -7158,7 +7198,7 @@
         <v>105</v>
       </c>
       <c r="I26" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -7247,13 +7287,13 @@
         <v>18</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C30" t="s">
         <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E30" s="4">
         <v>434.5</v>
@@ -7266,10 +7306,10 @@
         <v>434.5</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -7299,7 +7339,7 @@
         <v>135</v>
       </c>
       <c r="I31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -7329,7 +7369,7 @@
         <v>135</v>
       </c>
       <c r="I32" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -7359,7 +7399,7 @@
         <v>135</v>
       </c>
       <c r="I33" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -7389,7 +7429,7 @@
         <v>136</v>
       </c>
       <c r="I34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -7745,7 +7785,7 @@
         <v>101</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -7842,17 +7882,17 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>215</v>
+        <v>243</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>72</v>
       </c>
       <c r="C2" s="1">
-        <f>310*1.2/4600</f>
-        <v>8.0869565217391304E-2</v>
+        <f>500*1.2/4600</f>
+        <v>0.13043478260869565</v>
       </c>
       <c r="D2">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -7878,7 +7918,7 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit avant de faire l'intégration de l'ECS dans les charges
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1276" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5BCE6EF-3B86-4285-8B2D-14A1ABACB257}"/>
+  <xr:revisionPtr revIDLastSave="1297" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C1FEAFF-C718-4A32-9732-4AE22D2C289D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="415">
   <si>
     <t>Taxes</t>
   </si>
@@ -624,9 +624,6 @@
   </si>
   <si>
     <t>Prix unitaire du kWh</t>
-  </si>
-  <si>
-    <t>Atlantic Varmax 2 225</t>
   </si>
   <si>
     <t>Volume à chauffer en m3</t>
@@ -703,9 +700,6 @@
     <t>Description longue</t>
   </si>
   <si>
-    <t>Herz Firematic 130</t>
-  </si>
-  <si>
     <t>De 310€/t pour Gruchy à 500€/t pour Prochalor</t>
   </si>
   <si>
@@ -1283,6 +1277,27 @@
   </si>
   <si>
     <t>Prix de la tonne de granulés: Gruchy = 310€/t, CRAM = 392€/t (dans le simulateur) et Prochalor 500€/t - 1 tonne de granulés de bois = 4800-5000kWh</t>
+  </si>
+  <si>
+    <t>Herz Firematic 120</t>
+  </si>
+  <si>
+    <t>Atlantic Varmax 2 140</t>
+  </si>
+  <si>
+    <t>Unité</t>
+  </si>
+  <si>
+    <t>tonne de granulé</t>
+  </si>
+  <si>
+    <t>kWh</t>
+  </si>
+  <si>
+    <t>Prix de l'unité</t>
+  </si>
+  <si>
+    <t>kWh par unité</t>
   </si>
 </sst>
 </file>
@@ -1293,7 +1308,7 @@
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1304,6 +1319,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1348,7 +1369,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1367,13 +1388,52 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="30">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1431,30 +1491,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1725,6 +1761,48 @@
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1753,8 +1831,8 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1767,24 +1845,24 @@
     <sortCondition ref="A1:A180"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="25"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="25">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="24">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="24"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="22"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="21"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="20"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="19"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="17"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="15"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="14"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="20"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="18"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="17"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="16"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="15"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="14"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="13"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1797,17 +1875,17 @@
     <sortCondition ref="B1:B45"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="5">
       <calculatedColumnFormula>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1828,12 +1906,15 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:F3" totalsRowShown="0">
-  <autoFilter ref="A1:F3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:I3" totalsRowShown="0">
+  <autoFilter ref="A1:I3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
-    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="0" dataCellStyle="Currency"/>
+    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="29" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="2" dataCellStyle="Currency"/>
+    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix de l'unité" dataDxfId="1" dataCellStyle="Currency"/>
+    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="0" dataCellStyle="Currency"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="5" xr3:uid="{ED1B8FB3-6899-430D-BDC7-A9BDBA679526}" name="Ordre d'utilisation"/>
     <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
@@ -2136,7 +2217,7 @@
         <v>95</v>
       </c>
       <c r="F1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2144,7 +2225,7 @@
         <v>145</v>
       </c>
       <c r="B2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
@@ -2156,7 +2237,7 @@
         <v>35000</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2176,7 +2257,7 @@
         <v>27000</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2394,7 +2475,7 @@
         <v>2000</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2450,7 +2531,7 @@
         <v>1050</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2470,7 +2551,7 @@
         <v>1000</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2490,7 +2571,7 @@
         <v>1000</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="75" x14ac:dyDescent="0.25">
@@ -2510,7 +2591,7 @@
         <v>920</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -2530,7 +2611,7 @@
         <v>900</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2568,7 +2649,7 @@
         <v>750</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2606,7 +2687,7 @@
         <v>580</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2644,7 +2725,7 @@
         <v>450</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2664,7 +2745,7 @@
         <v>360</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2684,7 +2765,7 @@
         <v>320</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2704,7 +2785,7 @@
         <v>240</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2742,7 +2823,7 @@
         <v>90</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2766,16 +2847,16 @@
         <v>145</v>
       </c>
       <c r="B35" t="s">
+        <v>223</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D35" t="s">
+        <v>224</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="D35" t="s">
-        <v>226</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -2862,7 +2943,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C2">
         <v>462</v>
@@ -2876,7 +2957,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C3">
         <v>119</v>
@@ -2902,7 +2983,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C4">
         <v>83</v>
@@ -2928,7 +3009,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C5">
         <v>130</v>
@@ -2954,7 +3035,7 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -2980,7 +3061,7 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C7">
         <v>122</v>
@@ -3006,7 +3087,7 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C8">
         <v>55</v>
@@ -3032,7 +3113,7 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C9">
         <v>96</v>
@@ -3058,7 +3139,7 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C10">
         <v>123</v>
@@ -3084,7 +3165,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C11">
         <v>129</v>
@@ -3110,7 +3191,7 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C12">
         <v>58</v>
@@ -3136,7 +3217,7 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C13">
         <v>91</v>
@@ -3162,7 +3243,7 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C14" s="8">
         <v>86</v>
@@ -3196,7 +3277,7 @@
         <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C15">
         <v>94</v>
@@ -3222,7 +3303,7 @@
         <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C16">
         <v>60</v>
@@ -3248,7 +3329,7 @@
         <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C17">
         <v>162</v>
@@ -3274,7 +3355,7 @@
         <v>117</v>
       </c>
       <c r="B18" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C18">
         <v>202</v>
@@ -3300,7 +3381,7 @@
         <v>118</v>
       </c>
       <c r="B19" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C19">
         <v>294</v>
@@ -3326,7 +3407,7 @@
         <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C20">
         <v>81</v>
@@ -3352,7 +3433,7 @@
         <v>120</v>
       </c>
       <c r="B21" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C21">
         <v>115</v>
@@ -3378,7 +3459,7 @@
         <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C22">
         <v>112</v>
@@ -3404,7 +3485,7 @@
         <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C23">
         <v>83</v>
@@ -3430,7 +3511,7 @@
         <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C24">
         <v>118</v>
@@ -3456,7 +3537,7 @@
         <v>124</v>
       </c>
       <c r="B25" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C25">
         <v>117</v>
@@ -3482,7 +3563,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C26">
         <v>87</v>
@@ -3508,7 +3589,7 @@
         <v>126</v>
       </c>
       <c r="B27" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C27">
         <v>125</v>
@@ -3534,7 +3615,7 @@
         <v>127</v>
       </c>
       <c r="B28" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C28">
         <v>123</v>
@@ -3560,7 +3641,7 @@
         <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C29">
         <v>88</v>
@@ -3586,7 +3667,7 @@
         <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C30">
         <v>127</v>
@@ -3612,7 +3693,7 @@
         <v>130</v>
       </c>
       <c r="B31" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C31">
         <v>127</v>
@@ -3638,7 +3719,7 @@
         <v>132</v>
       </c>
       <c r="B32" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C32">
         <v>172</v>
@@ -3664,7 +3745,7 @@
         <v>133</v>
       </c>
       <c r="B33" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C33">
         <v>218</v>
@@ -3690,7 +3771,7 @@
         <v>134</v>
       </c>
       <c r="B34" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C34">
         <v>102</v>
@@ -3716,7 +3797,7 @@
         <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C35">
         <v>83</v>
@@ -3742,7 +3823,7 @@
         <v>201</v>
       </c>
       <c r="B36" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C36">
         <v>401</v>
@@ -3756,7 +3837,7 @@
         <v>202</v>
       </c>
       <c r="B37" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C37">
         <v>114</v>
@@ -3782,7 +3863,7 @@
         <v>203</v>
       </c>
       <c r="B38" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C38">
         <v>84</v>
@@ -3808,7 +3889,7 @@
         <v>204</v>
       </c>
       <c r="B39" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C39">
         <v>81</v>
@@ -3834,7 +3915,7 @@
         <v>205</v>
       </c>
       <c r="B40" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C40">
         <v>118</v>
@@ -3860,7 +3941,7 @@
         <v>206</v>
       </c>
       <c r="B41" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C41">
         <v>120</v>
@@ -3886,7 +3967,7 @@
         <v>207</v>
       </c>
       <c r="B42" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C42">
         <v>89</v>
@@ -3912,7 +3993,7 @@
         <v>208</v>
       </c>
       <c r="B43" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C43">
         <v>84</v>
@@ -3938,7 +4019,7 @@
         <v>209</v>
       </c>
       <c r="B44" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C44">
         <v>124</v>
@@ -3964,7 +4045,7 @@
         <v>210</v>
       </c>
       <c r="B45" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C45">
         <v>126</v>
@@ -3990,7 +4071,7 @@
         <v>211</v>
       </c>
       <c r="B46" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C46">
         <v>91</v>
@@ -4016,7 +4097,7 @@
         <v>212</v>
       </c>
       <c r="B47" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C47">
         <v>88</v>
@@ -4042,7 +4123,7 @@
         <v>213</v>
       </c>
       <c r="B48" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C48">
         <v>131</v>
@@ -4068,7 +4149,7 @@
         <v>214</v>
       </c>
       <c r="B49" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C49">
         <v>130</v>
@@ -4094,7 +4175,7 @@
         <v>215</v>
       </c>
       <c r="B50" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C50">
         <v>93</v>
@@ -4120,7 +4201,7 @@
         <v>216</v>
       </c>
       <c r="B51" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C51">
         <v>59</v>
@@ -4146,7 +4227,7 @@
         <v>217</v>
       </c>
       <c r="B52" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C52">
         <v>166</v>
@@ -4172,7 +4253,7 @@
         <v>218</v>
       </c>
       <c r="B53" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C53">
         <v>186</v>
@@ -4198,7 +4279,7 @@
         <v>219</v>
       </c>
       <c r="B54" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C54">
         <v>61</v>
@@ -4224,7 +4305,7 @@
         <v>220</v>
       </c>
       <c r="B55" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C55">
         <v>171</v>
@@ -4250,7 +4331,7 @@
         <v>221</v>
       </c>
       <c r="B56" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C56">
         <v>178</v>
@@ -4276,7 +4357,7 @@
         <v>222</v>
       </c>
       <c r="B57" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C57">
         <v>62</v>
@@ -4302,7 +4383,7 @@
         <v>223</v>
       </c>
       <c r="B58" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C58">
         <v>174</v>
@@ -4328,7 +4409,7 @@
         <v>224</v>
       </c>
       <c r="B59" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C59">
         <v>181</v>
@@ -4354,7 +4435,7 @@
         <v>225</v>
       </c>
       <c r="B60" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C60" s="8">
         <v>197</v>
@@ -4388,7 +4469,7 @@
         <v>301</v>
       </c>
       <c r="B61" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C61">
         <v>169</v>
@@ -4408,7 +4489,7 @@
         <v>302</v>
       </c>
       <c r="B62" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C62">
         <v>158</v>
@@ -4428,7 +4509,7 @@
         <v>303</v>
       </c>
       <c r="B63" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C63">
         <v>71</v>
@@ -4448,7 +4529,7 @@
         <v>305</v>
       </c>
       <c r="B64" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C64">
         <v>134</v>
@@ -4471,7 +4552,7 @@
         <v>306</v>
       </c>
       <c r="B65" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C65">
         <v>147</v>
@@ -4494,7 +4575,7 @@
         <v>307</v>
       </c>
       <c r="B66" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C66">
         <v>155</v>
@@ -4517,7 +4598,7 @@
         <v>308</v>
       </c>
       <c r="B67" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C67" s="8">
         <v>75</v>
@@ -4549,7 +4630,7 @@
         <v>310</v>
       </c>
       <c r="B68" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C68">
         <v>52</v>
@@ -4572,7 +4653,7 @@
         <v>311</v>
       </c>
       <c r="B69" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C69">
         <v>193</v>
@@ -4595,7 +4676,7 @@
         <v>312</v>
       </c>
       <c r="B70" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C70">
         <v>133</v>
@@ -4618,7 +4699,7 @@
         <v>313</v>
       </c>
       <c r="B71" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C71">
         <v>72</v>
@@ -4638,7 +4719,7 @@
         <v>314</v>
       </c>
       <c r="B72" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C72">
         <v>79</v>
@@ -4658,7 +4739,7 @@
         <v>315</v>
       </c>
       <c r="B73" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C73">
         <v>85</v>
@@ -4681,7 +4762,7 @@
         <v>316</v>
       </c>
       <c r="B74" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C74">
         <v>90</v>
@@ -4704,7 +4785,7 @@
         <v>401</v>
       </c>
       <c r="B75" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C75">
         <v>7</v>
@@ -4724,7 +4805,7 @@
         <v>402</v>
       </c>
       <c r="B76" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C76">
         <v>7</v>
@@ -4744,7 +4825,7 @@
         <v>403</v>
       </c>
       <c r="B77" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C77">
         <v>7</v>
@@ -4764,7 +4845,7 @@
         <v>404</v>
       </c>
       <c r="B78" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C78">
         <v>7</v>
@@ -4784,7 +4865,7 @@
         <v>405</v>
       </c>
       <c r="B79" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C79">
         <v>7</v>
@@ -4804,7 +4885,7 @@
         <v>406</v>
       </c>
       <c r="B80" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C80">
         <v>7</v>
@@ -4824,7 +4905,7 @@
         <v>407</v>
       </c>
       <c r="B81" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C81">
         <v>7</v>
@@ -4844,7 +4925,7 @@
         <v>408</v>
       </c>
       <c r="B82" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C82">
         <v>7</v>
@@ -4864,7 +4945,7 @@
         <v>409</v>
       </c>
       <c r="B83" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C83">
         <v>7</v>
@@ -4884,7 +4965,7 @@
         <v>410</v>
       </c>
       <c r="B84" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C84">
         <v>7</v>
@@ -4904,7 +4985,7 @@
         <v>411</v>
       </c>
       <c r="B85" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C85">
         <v>7</v>
@@ -4924,7 +5005,7 @@
         <v>412</v>
       </c>
       <c r="B86" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C86">
         <v>7</v>
@@ -4944,7 +5025,7 @@
         <v>413</v>
       </c>
       <c r="B87" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C87">
         <v>7</v>
@@ -4964,7 +5045,7 @@
         <v>414</v>
       </c>
       <c r="B88" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C88">
         <v>7</v>
@@ -4984,7 +5065,7 @@
         <v>415</v>
       </c>
       <c r="B89" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C89">
         <v>7</v>
@@ -5004,7 +5085,7 @@
         <v>416</v>
       </c>
       <c r="B90" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C90">
         <v>7</v>
@@ -5024,7 +5105,7 @@
         <v>417</v>
       </c>
       <c r="B91" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C91">
         <v>7</v>
@@ -5044,7 +5125,7 @@
         <v>418</v>
       </c>
       <c r="B92" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C92">
         <v>7</v>
@@ -5064,7 +5145,7 @@
         <v>419</v>
       </c>
       <c r="B93" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C93">
         <v>7</v>
@@ -5084,7 +5165,7 @@
         <v>420</v>
       </c>
       <c r="B94" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C94">
         <v>7</v>
@@ -5104,7 +5185,7 @@
         <v>421</v>
       </c>
       <c r="B95" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C95">
         <v>7</v>
@@ -5124,7 +5205,7 @@
         <v>422</v>
       </c>
       <c r="B96" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C96">
         <v>7</v>
@@ -5144,7 +5225,7 @@
         <v>423</v>
       </c>
       <c r="B97" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C97">
         <v>7</v>
@@ -5164,7 +5245,7 @@
         <v>424</v>
       </c>
       <c r="B98" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C98">
         <v>7</v>
@@ -5184,7 +5265,7 @@
         <v>425</v>
       </c>
       <c r="B99" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C99">
         <v>7</v>
@@ -5204,7 +5285,7 @@
         <v>426</v>
       </c>
       <c r="B100" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C100">
         <v>7</v>
@@ -5224,7 +5305,7 @@
         <v>427</v>
       </c>
       <c r="B101" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C101">
         <v>7</v>
@@ -5244,7 +5325,7 @@
         <v>428</v>
       </c>
       <c r="B102" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C102">
         <v>7</v>
@@ -5264,7 +5345,7 @@
         <v>429</v>
       </c>
       <c r="B103" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C103">
         <v>7</v>
@@ -5284,7 +5365,7 @@
         <v>430</v>
       </c>
       <c r="B104" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C104">
         <v>7</v>
@@ -5304,7 +5385,7 @@
         <v>431</v>
       </c>
       <c r="B105" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C105">
         <v>7</v>
@@ -5324,7 +5405,7 @@
         <v>432</v>
       </c>
       <c r="B106" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C106">
         <v>7</v>
@@ -5344,7 +5425,7 @@
         <v>433</v>
       </c>
       <c r="B107" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C107">
         <v>7</v>
@@ -5364,7 +5445,7 @@
         <v>434</v>
       </c>
       <c r="B108" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C108">
         <v>7</v>
@@ -5384,7 +5465,7 @@
         <v>435</v>
       </c>
       <c r="B109" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C109">
         <v>7</v>
@@ -5404,7 +5485,7 @@
         <v>436</v>
       </c>
       <c r="B110" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C110">
         <v>7</v>
@@ -5424,7 +5505,7 @@
         <v>437</v>
       </c>
       <c r="B111" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C111">
         <v>7</v>
@@ -5444,7 +5525,7 @@
         <v>438</v>
       </c>
       <c r="B112" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C112">
         <v>7</v>
@@ -5464,7 +5545,7 @@
         <v>439</v>
       </c>
       <c r="B113" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C113">
         <v>7</v>
@@ -5484,7 +5565,7 @@
         <v>440</v>
       </c>
       <c r="B114" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C114">
         <v>7</v>
@@ -5504,7 +5585,7 @@
         <v>441</v>
       </c>
       <c r="B115" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C115">
         <v>7</v>
@@ -5524,7 +5605,7 @@
         <v>442</v>
       </c>
       <c r="B116" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C116">
         <v>7</v>
@@ -5544,7 +5625,7 @@
         <v>443</v>
       </c>
       <c r="B117" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C117">
         <v>7</v>
@@ -5564,7 +5645,7 @@
         <v>444</v>
       </c>
       <c r="B118" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C118">
         <v>7</v>
@@ -5584,7 +5665,7 @@
         <v>445</v>
       </c>
       <c r="B119" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C119">
         <v>7</v>
@@ -5604,7 +5685,7 @@
         <v>446</v>
       </c>
       <c r="B120" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C120">
         <v>7</v>
@@ -5624,7 +5705,7 @@
         <v>447</v>
       </c>
       <c r="B121" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C121">
         <v>7</v>
@@ -5644,7 +5725,7 @@
         <v>448</v>
       </c>
       <c r="B122" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C122">
         <v>7</v>
@@ -5664,7 +5745,7 @@
         <v>449</v>
       </c>
       <c r="B123" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C123">
         <v>7</v>
@@ -5684,7 +5765,7 @@
         <v>450</v>
       </c>
       <c r="B124" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C124">
         <v>7</v>
@@ -5704,7 +5785,7 @@
         <v>451</v>
       </c>
       <c r="B125" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C125">
         <v>7</v>
@@ -5724,7 +5805,7 @@
         <v>452</v>
       </c>
       <c r="B126" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C126">
         <v>7</v>
@@ -5744,7 +5825,7 @@
         <v>453</v>
       </c>
       <c r="B127" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C127">
         <v>7</v>
@@ -5764,7 +5845,7 @@
         <v>454</v>
       </c>
       <c r="B128" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C128">
         <v>7</v>
@@ -5784,7 +5865,7 @@
         <v>455</v>
       </c>
       <c r="B129" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C129">
         <v>7</v>
@@ -5804,7 +5885,7 @@
         <v>456</v>
       </c>
       <c r="B130" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C130">
         <v>7</v>
@@ -5824,7 +5905,7 @@
         <v>457</v>
       </c>
       <c r="B131" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C131">
         <v>7</v>
@@ -5844,7 +5925,7 @@
         <v>458</v>
       </c>
       <c r="B132" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C132">
         <v>7</v>
@@ -5864,7 +5945,7 @@
         <v>459</v>
       </c>
       <c r="B133" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C133">
         <v>7</v>
@@ -5884,7 +5965,7 @@
         <v>460</v>
       </c>
       <c r="B134" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C134">
         <v>7</v>
@@ -5904,7 +5985,7 @@
         <v>461</v>
       </c>
       <c r="B135" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C135">
         <v>7</v>
@@ -5924,7 +6005,7 @@
         <v>462</v>
       </c>
       <c r="B136" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C136">
         <v>7</v>
@@ -5944,7 +6025,7 @@
         <v>463</v>
       </c>
       <c r="B137" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C137">
         <v>7</v>
@@ -5964,7 +6045,7 @@
         <v>464</v>
       </c>
       <c r="B138" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C138">
         <v>7</v>
@@ -5984,7 +6065,7 @@
         <v>465</v>
       </c>
       <c r="B139" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C139">
         <v>7</v>
@@ -6004,7 +6085,7 @@
         <v>466</v>
       </c>
       <c r="B140" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C140">
         <v>7</v>
@@ -6024,7 +6105,7 @@
         <v>467</v>
       </c>
       <c r="B141" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C141">
         <v>7</v>
@@ -6044,7 +6125,7 @@
         <v>468</v>
       </c>
       <c r="B142" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C142">
         <v>7</v>
@@ -6064,7 +6145,7 @@
         <v>469</v>
       </c>
       <c r="B143" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C143">
         <v>7</v>
@@ -6084,7 +6165,7 @@
         <v>470</v>
       </c>
       <c r="B144" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C144">
         <v>7</v>
@@ -6104,7 +6185,7 @@
         <v>471</v>
       </c>
       <c r="B145" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C145">
         <v>7</v>
@@ -6124,7 +6205,7 @@
         <v>472</v>
       </c>
       <c r="B146" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C146">
         <v>7</v>
@@ -6144,7 +6225,7 @@
         <v>473</v>
       </c>
       <c r="B147" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C147">
         <v>7</v>
@@ -6164,7 +6245,7 @@
         <v>474</v>
       </c>
       <c r="B148" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C148">
         <v>7</v>
@@ -6184,7 +6265,7 @@
         <v>475</v>
       </c>
       <c r="B149" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C149">
         <v>7</v>
@@ -6204,7 +6285,7 @@
         <v>476</v>
       </c>
       <c r="B150" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C150">
         <v>7</v>
@@ -6224,7 +6305,7 @@
         <v>477</v>
       </c>
       <c r="B151" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C151">
         <v>7</v>
@@ -6244,7 +6325,7 @@
         <v>478</v>
       </c>
       <c r="B152" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C152">
         <v>7</v>
@@ -6264,7 +6345,7 @@
         <v>479</v>
       </c>
       <c r="B153" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C153">
         <v>7</v>
@@ -6284,7 +6365,7 @@
         <v>480</v>
       </c>
       <c r="B154" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C154">
         <v>7</v>
@@ -6304,7 +6385,7 @@
         <v>481</v>
       </c>
       <c r="B155" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C155">
         <v>7</v>
@@ -6324,7 +6405,7 @@
         <v>482</v>
       </c>
       <c r="B156" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C156">
         <v>7</v>
@@ -6344,7 +6425,7 @@
         <v>483</v>
       </c>
       <c r="B157" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C157">
         <v>7</v>
@@ -6364,7 +6445,7 @@
         <v>484</v>
       </c>
       <c r="B158" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C158">
         <v>7</v>
@@ -6384,7 +6465,7 @@
         <v>485</v>
       </c>
       <c r="B159" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C159">
         <v>7</v>
@@ -6404,7 +6485,7 @@
         <v>486</v>
       </c>
       <c r="B160" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C160">
         <v>7</v>
@@ -6424,7 +6505,7 @@
         <v>487</v>
       </c>
       <c r="B161" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C161">
         <v>7</v>
@@ -6444,7 +6525,7 @@
         <v>488</v>
       </c>
       <c r="B162" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C162">
         <v>7</v>
@@ -6464,7 +6545,7 @@
         <v>489</v>
       </c>
       <c r="B163" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C163">
         <v>7</v>
@@ -6484,7 +6565,7 @@
         <v>490</v>
       </c>
       <c r="B164" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C164">
         <v>7</v>
@@ -6504,7 +6585,7 @@
         <v>491</v>
       </c>
       <c r="B165" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C165">
         <v>7</v>
@@ -6524,7 +6605,7 @@
         <v>492</v>
       </c>
       <c r="B166" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C166">
         <v>7</v>
@@ -6544,7 +6625,7 @@
         <v>493</v>
       </c>
       <c r="B167" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C167">
         <v>7</v>
@@ -6564,7 +6645,7 @@
         <v>494</v>
       </c>
       <c r="B168" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C168">
         <v>7</v>
@@ -6584,7 +6665,7 @@
         <v>495</v>
       </c>
       <c r="B169" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C169">
         <v>7</v>
@@ -6604,7 +6685,7 @@
         <v>496</v>
       </c>
       <c r="B170" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C170">
         <v>7</v>
@@ -6624,7 +6705,7 @@
         <v>497</v>
       </c>
       <c r="B171" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C171">
         <v>7</v>
@@ -6644,7 +6725,7 @@
         <v>498</v>
       </c>
       <c r="B172" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C172">
         <v>7</v>
@@ -6664,7 +6745,7 @@
         <v>499</v>
       </c>
       <c r="B173" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C173">
         <v>7</v>
@@ -6684,7 +6765,7 @@
         <v>500</v>
       </c>
       <c r="B174" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C174">
         <v>7</v>
@@ -6704,7 +6785,7 @@
         <v>501</v>
       </c>
       <c r="B175" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C175">
         <v>7</v>
@@ -6724,7 +6805,7 @@
         <v>502</v>
       </c>
       <c r="B176" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C176">
         <v>1</v>
@@ -6742,7 +6823,7 @@
         <v>503</v>
       </c>
       <c r="B177" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -6760,7 +6841,7 @@
         <v>504</v>
       </c>
       <c r="B178" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C178">
         <v>1</v>
@@ -6778,7 +6859,7 @@
         <v>505</v>
       </c>
       <c r="B179" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -6796,7 +6877,7 @@
         <v>506</v>
       </c>
       <c r="B180" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C180">
         <v>7</v>
@@ -6864,7 +6945,7 @@
         <v>136</v>
       </c>
       <c r="I1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -7197,7 +7278,7 @@
         <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -7227,7 +7308,7 @@
         <v>100</v>
       </c>
       <c r="I15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -7282,7 +7363,7 @@
         <v>16750</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -7290,7 +7371,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C18" t="s">
         <v>72</v>
@@ -7445,7 +7526,7 @@
         <v>103</v>
       </c>
       <c r="I23" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -7534,13 +7615,13 @@
         <v>18</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C27" t="s">
         <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E27" s="4">
         <v>434.5</v>
@@ -7553,10 +7634,10 @@
         <v>434.5</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -7586,7 +7667,7 @@
         <v>133</v>
       </c>
       <c r="I28" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -7616,7 +7697,7 @@
         <v>133</v>
       </c>
       <c r="I29" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -7646,7 +7727,7 @@
         <v>133</v>
       </c>
       <c r="I30" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -7676,7 +7757,7 @@
         <v>134</v>
       </c>
       <c r="I31" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -8032,7 +8113,7 @@
         <v>99</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -8070,10 +8151,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C1" t="s">
         <v>190</v>
@@ -8081,7 +8162,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B2">
         <f>5735*2.5</f>
@@ -8104,7 +8185,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
@@ -8112,10 +8193,13 @@
     <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" customWidth="1"/>
-    <col min="6" max="6" width="133.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="133.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>191</v>
       </c>
@@ -8125,19 +8209,28 @@
       <c r="C1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D1" t="s">
-        <v>200</v>
-      </c>
-      <c r="E1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>414</v>
+      </c>
+      <c r="G1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>216</v>
+        <v>408</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>70</v>
@@ -8146,19 +8239,28 @@
         <f>392*1.2/4900</f>
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="D2">
-        <v>130</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="E2" s="1">
+        <v>392</v>
+      </c>
+      <c r="F2" s="12">
+        <v>4900</v>
+      </c>
+      <c r="G2">
+        <v>120</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>409</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>194</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
@@ -8166,17 +8268,27 @@
       <c r="C3" s="1">
         <v>0.12559999999999999</v>
       </c>
-      <c r="D3">
-        <v>225</v>
-      </c>
-      <c r="E3">
+      <c r="D3" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.12559999999999999</v>
+      </c>
+      <c r="F3" s="12">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>140</v>
+      </c>
+      <c r="H3">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
-        <v>228</v>
+      <c r="I3" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Simulateur finaliser. Peut-être rajouter les pertes liées les heures de cycle de l'eau chaude dans les tuyaux
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1297" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C1FEAFF-C718-4A32-9732-4AE22D2C289D}"/>
+  <xr:revisionPtr revIDLastSave="1309" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20F1F1F2-522E-4F69-BF13-868435BCF306}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="416">
   <si>
     <t>Taxes</t>
   </si>
@@ -633,9 +633,6 @@
   </si>
   <si>
     <t>Terrasses de Gallieni</t>
-  </si>
-  <si>
-    <t>Ordre d'utilisation</t>
   </si>
   <si>
     <t>Contrat  P2, engagement sur 3 ans</t>
@@ -733,9 +730,6 @@
     <t>Le fonds travaux ALUR doit représenter 5% du budget provisionnel, mais les copropritété de résidence de moins de 5 ans en sont exemptés</t>
   </si>
   <si>
-    <t>Chaudière d'appoint au gaz 0,1256€ le kWh</t>
-  </si>
-  <si>
     <t>La facturation par Est Ensemble est progressive, gratuit jusqu'à 10m3, puis de 10 à 28 m³ = 1,1988 € HT / m³, de 28 à 86 m³ = 1,3320 € HT / m³, de 86 à 101 m³ = 1,3720 € HT / m³, de 101 à 131 m³ = 1,4200 € HT / m³, de 131 à 140 m³ = 1,4919 € HT / m³ et Plus de 140 m³ = 1,5366 € HT / m³. On rajoute la redevance (3,3€/m3) et la TVA (8%). Pour référence la consommation moyenne d'eau d'un adulte sur 1 an est de 55 m3.</t>
   </si>
   <si>
@@ -1298,6 +1292,15 @@
   </si>
   <si>
     <t>kWh par unité</t>
+  </si>
+  <si>
+    <t>Chaudière d'appoint au gaz à condensation 0,1256€ le kWh</t>
+  </si>
+  <si>
+    <t>Seuil de durée d'activation (mn)</t>
+  </si>
+  <si>
+    <t>Seuil de fonctionnement (%)</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1392,7 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1397,61 +1400,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="30">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1802,6 +1750,61 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1816,10 +1819,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:F35">
   <autoFilter ref="A1:F35" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1831,8 +1830,8 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1845,24 +1844,24 @@
     <sortCondition ref="A1:A180"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="22"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="24">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="21">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="18"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="17"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="16"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="15"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="13"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="17"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="16"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="13"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="12"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="11"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="10"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1875,17 +1874,17 @@
     <sortCondition ref="B1:B45"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="2">
       <calculatedColumnFormula>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1906,18 +1905,19 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:I3" totalsRowShown="0">
-  <autoFilter ref="A1:I3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}" name="Chauffage" displayName="Chauffage" ref="A1:J3" totalsRowShown="0">
+  <autoFilter ref="A1:J3" xr:uid="{587622F4-20CE-4A1D-A4F7-C9DCD51AF751}"/>
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
     <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="29" dataCellStyle="Currency"/>
-    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="2" dataCellStyle="Currency"/>
-    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix de l'unité" dataDxfId="1" dataCellStyle="Currency"/>
-    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="0" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="28" dataCellStyle="Currency"/>
+    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix de l'unité" dataDxfId="27" dataCellStyle="Currency"/>
+    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="26" dataCellStyle="Currency"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
-    <tableColumn id="5" xr3:uid="{ED1B8FB3-6899-430D-BDC7-A9BDBA679526}" name="Ordre d'utilisation"/>
     <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
+    <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (%)"/>
+    <tableColumn id="11" xr3:uid="{D0B5F61C-1D85-4C5E-A117-B774F88FE50E}" name="Seuil de durée d'activation (mn)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2217,7 +2217,7 @@
         <v>95</v>
       </c>
       <c r="F1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2225,7 +2225,7 @@
         <v>145</v>
       </c>
       <c r="B2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
@@ -2237,7 +2237,7 @@
         <v>35000</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2257,7 +2257,7 @@
         <v>27000</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2475,7 +2475,7 @@
         <v>2000</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2531,7 +2531,7 @@
         <v>1050</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2551,7 +2551,7 @@
         <v>1000</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2571,7 +2571,7 @@
         <v>1000</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="75" x14ac:dyDescent="0.25">
@@ -2591,7 +2591,7 @@
         <v>920</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -2611,7 +2611,7 @@
         <v>900</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2649,7 +2649,7 @@
         <v>750</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2687,7 +2687,7 @@
         <v>580</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2725,7 +2725,7 @@
         <v>450</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2745,7 +2745,7 @@
         <v>360</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2765,7 +2765,7 @@
         <v>320</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2785,7 +2785,7 @@
         <v>240</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2823,7 +2823,7 @@
         <v>90</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2847,16 +2847,16 @@
         <v>145</v>
       </c>
       <c r="B35" t="s">
+        <v>222</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D35" t="s">
         <v>223</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="F35" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -2943,7 +2943,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C2">
         <v>462</v>
@@ -2957,7 +2957,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C3">
         <v>119</v>
@@ -2983,7 +2983,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C4">
         <v>83</v>
@@ -3009,7 +3009,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C5">
         <v>130</v>
@@ -3035,7 +3035,7 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -3061,7 +3061,7 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C7">
         <v>122</v>
@@ -3087,7 +3087,7 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C8">
         <v>55</v>
@@ -3113,7 +3113,7 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C9">
         <v>96</v>
@@ -3139,7 +3139,7 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C10">
         <v>123</v>
@@ -3165,7 +3165,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C11">
         <v>129</v>
@@ -3191,7 +3191,7 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C12">
         <v>58</v>
@@ -3217,7 +3217,7 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C13">
         <v>91</v>
@@ -3243,7 +3243,7 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C14" s="8">
         <v>86</v>
@@ -3277,7 +3277,7 @@
         <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C15">
         <v>94</v>
@@ -3303,7 +3303,7 @@
         <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C16">
         <v>60</v>
@@ -3329,7 +3329,7 @@
         <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C17">
         <v>162</v>
@@ -3355,7 +3355,7 @@
         <v>117</v>
       </c>
       <c r="B18" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C18">
         <v>202</v>
@@ -3381,7 +3381,7 @@
         <v>118</v>
       </c>
       <c r="B19" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C19">
         <v>294</v>
@@ -3407,7 +3407,7 @@
         <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C20">
         <v>81</v>
@@ -3433,7 +3433,7 @@
         <v>120</v>
       </c>
       <c r="B21" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C21">
         <v>115</v>
@@ -3459,7 +3459,7 @@
         <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C22">
         <v>112</v>
@@ -3485,7 +3485,7 @@
         <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C23">
         <v>83</v>
@@ -3511,7 +3511,7 @@
         <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C24">
         <v>118</v>
@@ -3537,7 +3537,7 @@
         <v>124</v>
       </c>
       <c r="B25" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C25">
         <v>117</v>
@@ -3563,7 +3563,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C26">
         <v>87</v>
@@ -3589,7 +3589,7 @@
         <v>126</v>
       </c>
       <c r="B27" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C27">
         <v>125</v>
@@ -3615,7 +3615,7 @@
         <v>127</v>
       </c>
       <c r="B28" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C28">
         <v>123</v>
@@ -3641,7 +3641,7 @@
         <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C29">
         <v>88</v>
@@ -3667,7 +3667,7 @@
         <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C30">
         <v>127</v>
@@ -3693,7 +3693,7 @@
         <v>130</v>
       </c>
       <c r="B31" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C31">
         <v>127</v>
@@ -3719,7 +3719,7 @@
         <v>132</v>
       </c>
       <c r="B32" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C32">
         <v>172</v>
@@ -3745,7 +3745,7 @@
         <v>133</v>
       </c>
       <c r="B33" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C33">
         <v>218</v>
@@ -3771,7 +3771,7 @@
         <v>134</v>
       </c>
       <c r="B34" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C34">
         <v>102</v>
@@ -3797,7 +3797,7 @@
         <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C35">
         <v>83</v>
@@ -3823,7 +3823,7 @@
         <v>201</v>
       </c>
       <c r="B36" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C36">
         <v>401</v>
@@ -3837,7 +3837,7 @@
         <v>202</v>
       </c>
       <c r="B37" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C37">
         <v>114</v>
@@ -3863,7 +3863,7 @@
         <v>203</v>
       </c>
       <c r="B38" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C38">
         <v>84</v>
@@ -3889,7 +3889,7 @@
         <v>204</v>
       </c>
       <c r="B39" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C39">
         <v>81</v>
@@ -3915,7 +3915,7 @@
         <v>205</v>
       </c>
       <c r="B40" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C40">
         <v>118</v>
@@ -3941,7 +3941,7 @@
         <v>206</v>
       </c>
       <c r="B41" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C41">
         <v>120</v>
@@ -3967,7 +3967,7 @@
         <v>207</v>
       </c>
       <c r="B42" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C42">
         <v>89</v>
@@ -3993,7 +3993,7 @@
         <v>208</v>
       </c>
       <c r="B43" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C43">
         <v>84</v>
@@ -4019,7 +4019,7 @@
         <v>209</v>
       </c>
       <c r="B44" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C44">
         <v>124</v>
@@ -4045,7 +4045,7 @@
         <v>210</v>
       </c>
       <c r="B45" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C45">
         <v>126</v>
@@ -4071,7 +4071,7 @@
         <v>211</v>
       </c>
       <c r="B46" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C46">
         <v>91</v>
@@ -4097,7 +4097,7 @@
         <v>212</v>
       </c>
       <c r="B47" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C47">
         <v>88</v>
@@ -4123,7 +4123,7 @@
         <v>213</v>
       </c>
       <c r="B48" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C48">
         <v>131</v>
@@ -4149,7 +4149,7 @@
         <v>214</v>
       </c>
       <c r="B49" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C49">
         <v>130</v>
@@ -4175,7 +4175,7 @@
         <v>215</v>
       </c>
       <c r="B50" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C50">
         <v>93</v>
@@ -4201,7 +4201,7 @@
         <v>216</v>
       </c>
       <c r="B51" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C51">
         <v>59</v>
@@ -4227,7 +4227,7 @@
         <v>217</v>
       </c>
       <c r="B52" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C52">
         <v>166</v>
@@ -4253,7 +4253,7 @@
         <v>218</v>
       </c>
       <c r="B53" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C53">
         <v>186</v>
@@ -4279,7 +4279,7 @@
         <v>219</v>
       </c>
       <c r="B54" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C54">
         <v>61</v>
@@ -4305,7 +4305,7 @@
         <v>220</v>
       </c>
       <c r="B55" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C55">
         <v>171</v>
@@ -4331,7 +4331,7 @@
         <v>221</v>
       </c>
       <c r="B56" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C56">
         <v>178</v>
@@ -4357,7 +4357,7 @@
         <v>222</v>
       </c>
       <c r="B57" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C57">
         <v>62</v>
@@ -4383,7 +4383,7 @@
         <v>223</v>
       </c>
       <c r="B58" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C58">
         <v>174</v>
@@ -4409,7 +4409,7 @@
         <v>224</v>
       </c>
       <c r="B59" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C59">
         <v>181</v>
@@ -4435,7 +4435,7 @@
         <v>225</v>
       </c>
       <c r="B60" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C60" s="8">
         <v>197</v>
@@ -4469,7 +4469,7 @@
         <v>301</v>
       </c>
       <c r="B61" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C61">
         <v>169</v>
@@ -4489,7 +4489,7 @@
         <v>302</v>
       </c>
       <c r="B62" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C62">
         <v>158</v>
@@ -4509,7 +4509,7 @@
         <v>303</v>
       </c>
       <c r="B63" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C63">
         <v>71</v>
@@ -4529,7 +4529,7 @@
         <v>305</v>
       </c>
       <c r="B64" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C64">
         <v>134</v>
@@ -4552,7 +4552,7 @@
         <v>306</v>
       </c>
       <c r="B65" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C65">
         <v>147</v>
@@ -4575,7 +4575,7 @@
         <v>307</v>
       </c>
       <c r="B66" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C66">
         <v>155</v>
@@ -4598,7 +4598,7 @@
         <v>308</v>
       </c>
       <c r="B67" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C67" s="8">
         <v>75</v>
@@ -4630,7 +4630,7 @@
         <v>310</v>
       </c>
       <c r="B68" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C68">
         <v>52</v>
@@ -4653,7 +4653,7 @@
         <v>311</v>
       </c>
       <c r="B69" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C69">
         <v>193</v>
@@ -4676,7 +4676,7 @@
         <v>312</v>
       </c>
       <c r="B70" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C70">
         <v>133</v>
@@ -4699,7 +4699,7 @@
         <v>313</v>
       </c>
       <c r="B71" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C71">
         <v>72</v>
@@ -4719,7 +4719,7 @@
         <v>314</v>
       </c>
       <c r="B72" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C72">
         <v>79</v>
@@ -4739,7 +4739,7 @@
         <v>315</v>
       </c>
       <c r="B73" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C73">
         <v>85</v>
@@ -4762,7 +4762,7 @@
         <v>316</v>
       </c>
       <c r="B74" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C74">
         <v>90</v>
@@ -4785,7 +4785,7 @@
         <v>401</v>
       </c>
       <c r="B75" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C75">
         <v>7</v>
@@ -4805,7 +4805,7 @@
         <v>402</v>
       </c>
       <c r="B76" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C76">
         <v>7</v>
@@ -4825,7 +4825,7 @@
         <v>403</v>
       </c>
       <c r="B77" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C77">
         <v>7</v>
@@ -4845,7 +4845,7 @@
         <v>404</v>
       </c>
       <c r="B78" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C78">
         <v>7</v>
@@ -4865,7 +4865,7 @@
         <v>405</v>
       </c>
       <c r="B79" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C79">
         <v>7</v>
@@ -4885,7 +4885,7 @@
         <v>406</v>
       </c>
       <c r="B80" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C80">
         <v>7</v>
@@ -4905,7 +4905,7 @@
         <v>407</v>
       </c>
       <c r="B81" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C81">
         <v>7</v>
@@ -4925,7 +4925,7 @@
         <v>408</v>
       </c>
       <c r="B82" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C82">
         <v>7</v>
@@ -4945,7 +4945,7 @@
         <v>409</v>
       </c>
       <c r="B83" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C83">
         <v>7</v>
@@ -4965,7 +4965,7 @@
         <v>410</v>
       </c>
       <c r="B84" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C84">
         <v>7</v>
@@ -4985,7 +4985,7 @@
         <v>411</v>
       </c>
       <c r="B85" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C85">
         <v>7</v>
@@ -5005,7 +5005,7 @@
         <v>412</v>
       </c>
       <c r="B86" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C86">
         <v>7</v>
@@ -5025,7 +5025,7 @@
         <v>413</v>
       </c>
       <c r="B87" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C87">
         <v>7</v>
@@ -5045,7 +5045,7 @@
         <v>414</v>
       </c>
       <c r="B88" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C88">
         <v>7</v>
@@ -5065,7 +5065,7 @@
         <v>415</v>
       </c>
       <c r="B89" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C89">
         <v>7</v>
@@ -5085,7 +5085,7 @@
         <v>416</v>
       </c>
       <c r="B90" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C90">
         <v>7</v>
@@ -5105,7 +5105,7 @@
         <v>417</v>
       </c>
       <c r="B91" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C91">
         <v>7</v>
@@ -5125,7 +5125,7 @@
         <v>418</v>
       </c>
       <c r="B92" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C92">
         <v>7</v>
@@ -5145,7 +5145,7 @@
         <v>419</v>
       </c>
       <c r="B93" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C93">
         <v>7</v>
@@ -5165,7 +5165,7 @@
         <v>420</v>
       </c>
       <c r="B94" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C94">
         <v>7</v>
@@ -5185,7 +5185,7 @@
         <v>421</v>
       </c>
       <c r="B95" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C95">
         <v>7</v>
@@ -5205,7 +5205,7 @@
         <v>422</v>
       </c>
       <c r="B96" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C96">
         <v>7</v>
@@ -5225,7 +5225,7 @@
         <v>423</v>
       </c>
       <c r="B97" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C97">
         <v>7</v>
@@ -5245,7 +5245,7 @@
         <v>424</v>
       </c>
       <c r="B98" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C98">
         <v>7</v>
@@ -5265,7 +5265,7 @@
         <v>425</v>
       </c>
       <c r="B99" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C99">
         <v>7</v>
@@ -5285,7 +5285,7 @@
         <v>426</v>
       </c>
       <c r="B100" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C100">
         <v>7</v>
@@ -5305,7 +5305,7 @@
         <v>427</v>
       </c>
       <c r="B101" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C101">
         <v>7</v>
@@ -5325,7 +5325,7 @@
         <v>428</v>
       </c>
       <c r="B102" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C102">
         <v>7</v>
@@ -5345,7 +5345,7 @@
         <v>429</v>
       </c>
       <c r="B103" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C103">
         <v>7</v>
@@ -5365,7 +5365,7 @@
         <v>430</v>
       </c>
       <c r="B104" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C104">
         <v>7</v>
@@ -5385,7 +5385,7 @@
         <v>431</v>
       </c>
       <c r="B105" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C105">
         <v>7</v>
@@ -5405,7 +5405,7 @@
         <v>432</v>
       </c>
       <c r="B106" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C106">
         <v>7</v>
@@ -5425,7 +5425,7 @@
         <v>433</v>
       </c>
       <c r="B107" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C107">
         <v>7</v>
@@ -5445,7 +5445,7 @@
         <v>434</v>
       </c>
       <c r="B108" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C108">
         <v>7</v>
@@ -5465,7 +5465,7 @@
         <v>435</v>
       </c>
       <c r="B109" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C109">
         <v>7</v>
@@ -5485,7 +5485,7 @@
         <v>436</v>
       </c>
       <c r="B110" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C110">
         <v>7</v>
@@ -5505,7 +5505,7 @@
         <v>437</v>
       </c>
       <c r="B111" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C111">
         <v>7</v>
@@ -5525,7 +5525,7 @@
         <v>438</v>
       </c>
       <c r="B112" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C112">
         <v>7</v>
@@ -5545,7 +5545,7 @@
         <v>439</v>
       </c>
       <c r="B113" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C113">
         <v>7</v>
@@ -5565,7 +5565,7 @@
         <v>440</v>
       </c>
       <c r="B114" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C114">
         <v>7</v>
@@ -5585,7 +5585,7 @@
         <v>441</v>
       </c>
       <c r="B115" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C115">
         <v>7</v>
@@ -5605,7 +5605,7 @@
         <v>442</v>
       </c>
       <c r="B116" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C116">
         <v>7</v>
@@ -5625,7 +5625,7 @@
         <v>443</v>
       </c>
       <c r="B117" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C117">
         <v>7</v>
@@ -5645,7 +5645,7 @@
         <v>444</v>
       </c>
       <c r="B118" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C118">
         <v>7</v>
@@ -5665,7 +5665,7 @@
         <v>445</v>
       </c>
       <c r="B119" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C119">
         <v>7</v>
@@ -5685,7 +5685,7 @@
         <v>446</v>
       </c>
       <c r="B120" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C120">
         <v>7</v>
@@ -5705,7 +5705,7 @@
         <v>447</v>
       </c>
       <c r="B121" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C121">
         <v>7</v>
@@ -5725,7 +5725,7 @@
         <v>448</v>
       </c>
       <c r="B122" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C122">
         <v>7</v>
@@ -5745,7 +5745,7 @@
         <v>449</v>
       </c>
       <c r="B123" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C123">
         <v>7</v>
@@ -5765,7 +5765,7 @@
         <v>450</v>
       </c>
       <c r="B124" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C124">
         <v>7</v>
@@ -5785,7 +5785,7 @@
         <v>451</v>
       </c>
       <c r="B125" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C125">
         <v>7</v>
@@ -5805,7 +5805,7 @@
         <v>452</v>
       </c>
       <c r="B126" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C126">
         <v>7</v>
@@ -5825,7 +5825,7 @@
         <v>453</v>
       </c>
       <c r="B127" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C127">
         <v>7</v>
@@ -5845,7 +5845,7 @@
         <v>454</v>
       </c>
       <c r="B128" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C128">
         <v>7</v>
@@ -5865,7 +5865,7 @@
         <v>455</v>
       </c>
       <c r="B129" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C129">
         <v>7</v>
@@ -5885,7 +5885,7 @@
         <v>456</v>
       </c>
       <c r="B130" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C130">
         <v>7</v>
@@ -5905,7 +5905,7 @@
         <v>457</v>
       </c>
       <c r="B131" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C131">
         <v>7</v>
@@ -5925,7 +5925,7 @@
         <v>458</v>
       </c>
       <c r="B132" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C132">
         <v>7</v>
@@ -5945,7 +5945,7 @@
         <v>459</v>
       </c>
       <c r="B133" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C133">
         <v>7</v>
@@ -5965,7 +5965,7 @@
         <v>460</v>
       </c>
       <c r="B134" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C134">
         <v>7</v>
@@ -5985,7 +5985,7 @@
         <v>461</v>
       </c>
       <c r="B135" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C135">
         <v>7</v>
@@ -6005,7 +6005,7 @@
         <v>462</v>
       </c>
       <c r="B136" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C136">
         <v>7</v>
@@ -6025,7 +6025,7 @@
         <v>463</v>
       </c>
       <c r="B137" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C137">
         <v>7</v>
@@ -6045,7 +6045,7 @@
         <v>464</v>
       </c>
       <c r="B138" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C138">
         <v>7</v>
@@ -6065,7 +6065,7 @@
         <v>465</v>
       </c>
       <c r="B139" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C139">
         <v>7</v>
@@ -6085,7 +6085,7 @@
         <v>466</v>
       </c>
       <c r="B140" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C140">
         <v>7</v>
@@ -6105,7 +6105,7 @@
         <v>467</v>
       </c>
       <c r="B141" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C141">
         <v>7</v>
@@ -6125,7 +6125,7 @@
         <v>468</v>
       </c>
       <c r="B142" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C142">
         <v>7</v>
@@ -6145,7 +6145,7 @@
         <v>469</v>
       </c>
       <c r="B143" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C143">
         <v>7</v>
@@ -6165,7 +6165,7 @@
         <v>470</v>
       </c>
       <c r="B144" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C144">
         <v>7</v>
@@ -6185,7 +6185,7 @@
         <v>471</v>
       </c>
       <c r="B145" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C145">
         <v>7</v>
@@ -6205,7 +6205,7 @@
         <v>472</v>
       </c>
       <c r="B146" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C146">
         <v>7</v>
@@ -6225,7 +6225,7 @@
         <v>473</v>
       </c>
       <c r="B147" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C147">
         <v>7</v>
@@ -6245,7 +6245,7 @@
         <v>474</v>
       </c>
       <c r="B148" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C148">
         <v>7</v>
@@ -6265,7 +6265,7 @@
         <v>475</v>
       </c>
       <c r="B149" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C149">
         <v>7</v>
@@ -6285,7 +6285,7 @@
         <v>476</v>
       </c>
       <c r="B150" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C150">
         <v>7</v>
@@ -6305,7 +6305,7 @@
         <v>477</v>
       </c>
       <c r="B151" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C151">
         <v>7</v>
@@ -6325,7 +6325,7 @@
         <v>478</v>
       </c>
       <c r="B152" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C152">
         <v>7</v>
@@ -6345,7 +6345,7 @@
         <v>479</v>
       </c>
       <c r="B153" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C153">
         <v>7</v>
@@ -6365,7 +6365,7 @@
         <v>480</v>
       </c>
       <c r="B154" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C154">
         <v>7</v>
@@ -6385,7 +6385,7 @@
         <v>481</v>
       </c>
       <c r="B155" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C155">
         <v>7</v>
@@ -6405,7 +6405,7 @@
         <v>482</v>
       </c>
       <c r="B156" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C156">
         <v>7</v>
@@ -6425,7 +6425,7 @@
         <v>483</v>
       </c>
       <c r="B157" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C157">
         <v>7</v>
@@ -6445,7 +6445,7 @@
         <v>484</v>
       </c>
       <c r="B158" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C158">
         <v>7</v>
@@ -6465,7 +6465,7 @@
         <v>485</v>
       </c>
       <c r="B159" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C159">
         <v>7</v>
@@ -6485,7 +6485,7 @@
         <v>486</v>
       </c>
       <c r="B160" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C160">
         <v>7</v>
@@ -6505,7 +6505,7 @@
         <v>487</v>
       </c>
       <c r="B161" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C161">
         <v>7</v>
@@ -6525,7 +6525,7 @@
         <v>488</v>
       </c>
       <c r="B162" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C162">
         <v>7</v>
@@ -6545,7 +6545,7 @@
         <v>489</v>
       </c>
       <c r="B163" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C163">
         <v>7</v>
@@ -6565,7 +6565,7 @@
         <v>490</v>
       </c>
       <c r="B164" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C164">
         <v>7</v>
@@ -6585,7 +6585,7 @@
         <v>491</v>
       </c>
       <c r="B165" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C165">
         <v>7</v>
@@ -6605,7 +6605,7 @@
         <v>492</v>
       </c>
       <c r="B166" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C166">
         <v>7</v>
@@ -6625,7 +6625,7 @@
         <v>493</v>
       </c>
       <c r="B167" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C167">
         <v>7</v>
@@ -6645,7 +6645,7 @@
         <v>494</v>
       </c>
       <c r="B168" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C168">
         <v>7</v>
@@ -6665,7 +6665,7 @@
         <v>495</v>
       </c>
       <c r="B169" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C169">
         <v>7</v>
@@ -6685,7 +6685,7 @@
         <v>496</v>
       </c>
       <c r="B170" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C170">
         <v>7</v>
@@ -6705,7 +6705,7 @@
         <v>497</v>
       </c>
       <c r="B171" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C171">
         <v>7</v>
@@ -6725,7 +6725,7 @@
         <v>498</v>
       </c>
       <c r="B172" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C172">
         <v>7</v>
@@ -6745,7 +6745,7 @@
         <v>499</v>
       </c>
       <c r="B173" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C173">
         <v>7</v>
@@ -6765,7 +6765,7 @@
         <v>500</v>
       </c>
       <c r="B174" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C174">
         <v>7</v>
@@ -6785,7 +6785,7 @@
         <v>501</v>
       </c>
       <c r="B175" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C175">
         <v>7</v>
@@ -6805,7 +6805,7 @@
         <v>502</v>
       </c>
       <c r="B176" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C176">
         <v>1</v>
@@ -6823,7 +6823,7 @@
         <v>503</v>
       </c>
       <c r="B177" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -6841,7 +6841,7 @@
         <v>504</v>
       </c>
       <c r="B178" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C178">
         <v>1</v>
@@ -6859,7 +6859,7 @@
         <v>505</v>
       </c>
       <c r="B179" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -6877,7 +6877,7 @@
         <v>506</v>
       </c>
       <c r="B180" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C180">
         <v>7</v>
@@ -6945,7 +6945,7 @@
         <v>136</v>
       </c>
       <c r="I1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -7278,7 +7278,7 @@
         <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -7308,7 +7308,7 @@
         <v>100</v>
       </c>
       <c r="I15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -7363,7 +7363,7 @@
         <v>16750</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -7371,7 +7371,7 @@
         <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C18" t="s">
         <v>72</v>
@@ -7526,7 +7526,7 @@
         <v>103</v>
       </c>
       <c r="I23" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -7615,13 +7615,13 @@
         <v>18</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C27" t="s">
         <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E27" s="4">
         <v>434.5</v>
@@ -7634,10 +7634,10 @@
         <v>434.5</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -7667,7 +7667,7 @@
         <v>133</v>
       </c>
       <c r="I28" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -7697,7 +7697,7 @@
         <v>133</v>
       </c>
       <c r="I29" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -7727,7 +7727,7 @@
         <v>133</v>
       </c>
       <c r="I30" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -7757,7 +7757,7 @@
         <v>134</v>
       </c>
       <c r="I31" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -8113,7 +8113,7 @@
         <v>99</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -8185,7 +8185,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
@@ -8193,13 +8193,14 @@
     <col min="3" max="3" width="21.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="133.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="133.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.7109375" customWidth="1"/>
+    <col min="10" max="10" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>191</v>
       </c>
@@ -8210,27 +8211,30 @@
         <v>193</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="F1" s="12" t="s">
+        <v>412</v>
+      </c>
+      <c r="G1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I1" t="s">
+        <v>415</v>
+      </c>
+      <c r="J1" t="s">
         <v>414</v>
       </c>
-      <c r="G1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H1" t="s">
-        <v>197</v>
-      </c>
-      <c r="I1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>70</v>
@@ -8240,7 +8244,7 @@
         <v>9.6000000000000002E-2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E2" s="1">
         <v>392</v>
@@ -8251,16 +8255,19 @@
       <c r="G2">
         <v>120</v>
       </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="H2" t="s">
+        <v>405</v>
+      </c>
+      <c r="I2" s="13">
+        <v>0.3</v>
+      </c>
+      <c r="J2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>407</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>409</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
@@ -8269,7 +8276,7 @@
         <v>0.12559999999999999</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E3" s="1">
         <v>0.12559999999999999</v>
@@ -8280,18 +8287,22 @@
       <c r="G3">
         <v>140</v>
       </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3" t="s">
-        <v>226</v>
+      <c r="H3" t="s">
+        <v>413</v>
+      </c>
+      <c r="I3" s="13">
+        <v>0.08</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout prix de l'unite, expander du tableau
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1309" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20F1F1F2-522E-4F69-BF13-868435BCF306}"/>
+  <xr:revisionPtr revIDLastSave="1315" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD65BE4F-F1BF-4F83-BAED-91D17FA905CE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="404">
   <si>
     <t>Taxes</t>
   </si>
@@ -551,30 +551,6 @@
     <t>Electricité du batiment 3</t>
   </si>
   <si>
-    <t>Fourniture de granulé de bois</t>
-  </si>
-  <si>
-    <t>Fourniture de gaz</t>
-  </si>
-  <si>
-    <t>Chaudière biomasse à pleine capacité</t>
-  </si>
-  <si>
-    <t>Appoint au gaz léger</t>
-  </si>
-  <si>
-    <t>Appoint au gaz pour augmenter la température</t>
-  </si>
-  <si>
-    <t>Appoint au gaz pour un hiver rude</t>
-  </si>
-  <si>
-    <t>Chaudière biomasse en fonctionnement partiel</t>
-  </si>
-  <si>
-    <t>Chaudière biomasse en fonctionnement normal</t>
-  </si>
-  <si>
     <t>Tantièmes ascenseur 3</t>
   </si>
   <si>
@@ -588,18 +564,6 @@
   </si>
   <si>
     <t>Syndic fourcette moyenne</t>
-  </si>
-  <si>
-    <t>2 - Consommation pour un hiver doux</t>
-  </si>
-  <si>
-    <t>1 - Consommation pour un hiver très doux</t>
-  </si>
-  <si>
-    <t>3 - Consommation pour un hiver normal</t>
-  </si>
-  <si>
-    <t>4 - Consommation pour un hiver rude</t>
   </si>
   <si>
     <t>Tantièmes Stationnement</t>
@@ -1285,9 +1249,6 @@
     <t>tonne de granulé</t>
   </si>
   <si>
-    <t>kWh</t>
-  </si>
-  <si>
     <t>Prix de l'unité</t>
   </si>
   <si>
@@ -1301,6 +1262,9 @@
   </si>
   <si>
     <t>Seuil de fonctionnement (%)</t>
+  </si>
+  <si>
+    <t>kWh de gaz</t>
   </si>
 </sst>
 </file>
@@ -1395,9 +1359,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="30">
     <dxf>
@@ -1819,6 +1783,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:F35">
   <autoFilter ref="A1:F35" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1868,10 +1836,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I45" totalsRowShown="0">
-  <autoFilter ref="A1:I45" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H45">
-    <sortCondition ref="B1:B45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I37" totalsRowShown="0">
+  <autoFilter ref="A1:I37" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H37">
+    <sortCondition ref="B1:B37"/>
   </sortState>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="7"/>
@@ -1910,10 +1878,10 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
-    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="29" dataCellStyle="Currency"/>
-    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="28" dataCellStyle="Currency"/>
-    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix de l'unité" dataDxfId="27" dataCellStyle="Currency"/>
-    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="26" dataCellStyle="Currency"/>
+    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix de l'unité" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="26"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
     <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (%)"/>
@@ -2190,7 +2158,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:F35"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -2202,10 +2170,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B1" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C1" t="s">
         <v>136</v>
@@ -2217,7 +2185,7 @@
         <v>95</v>
       </c>
       <c r="F1" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2225,7 +2193,7 @@
         <v>145</v>
       </c>
       <c r="B2" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
@@ -2237,7 +2205,7 @@
         <v>35000</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2257,7 +2225,7 @@
         <v>27000</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2442,7 +2410,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
         <v>88</v>
@@ -2475,7 +2443,7 @@
         <v>2000</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2498,7 +2466,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B17" t="s">
         <v>89</v>
@@ -2531,7 +2499,7 @@
         <v>1050</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -2551,7 +2519,7 @@
         <v>1000</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2571,7 +2539,7 @@
         <v>1000</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="75" x14ac:dyDescent="0.25">
@@ -2591,7 +2559,7 @@
         <v>920</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -2611,7 +2579,7 @@
         <v>900</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2649,7 +2617,7 @@
         <v>750</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2687,7 +2655,7 @@
         <v>580</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2710,7 +2678,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B28" t="s">
         <v>73</v>
@@ -2725,12 +2693,12 @@
         <v>450</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B29" t="s">
         <v>76</v>
@@ -2745,12 +2713,12 @@
         <v>360</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B30" t="s">
         <v>75</v>
@@ -2765,7 +2733,7 @@
         <v>320</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2785,7 +2753,7 @@
         <v>240</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2808,7 +2776,7 @@
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B33" t="s">
         <v>74</v>
@@ -2823,7 +2791,7 @@
         <v>90</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2847,16 +2815,16 @@
         <v>145</v>
       </c>
       <c r="B35" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="D35" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2873,7 +2841,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:P180"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="54.85546875" bestFit="1" customWidth="1"/>
@@ -2908,7 +2876,7 @@
         <v>148</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>149</v>
@@ -2935,7 +2903,7 @@
         <v>156</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -2943,7 +2911,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="C2">
         <v>462</v>
@@ -2957,7 +2925,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="C3">
         <v>119</v>
@@ -2983,7 +2951,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="C4">
         <v>83</v>
@@ -3009,7 +2977,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="C5">
         <v>130</v>
@@ -3035,7 +3003,7 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -3061,7 +3029,7 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="C7">
         <v>122</v>
@@ -3087,7 +3055,7 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="C8">
         <v>55</v>
@@ -3113,7 +3081,7 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="C9">
         <v>96</v>
@@ -3139,7 +3107,7 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="C10">
         <v>123</v>
@@ -3165,7 +3133,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="C11">
         <v>129</v>
@@ -3191,7 +3159,7 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="C12">
         <v>58</v>
@@ -3217,7 +3185,7 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="C13">
         <v>91</v>
@@ -3243,7 +3211,7 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="C14" s="8">
         <v>86</v>
@@ -3277,7 +3245,7 @@
         <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="C15">
         <v>94</v>
@@ -3303,7 +3271,7 @@
         <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="C16">
         <v>60</v>
@@ -3329,7 +3297,7 @@
         <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="C17">
         <v>162</v>
@@ -3355,7 +3323,7 @@
         <v>117</v>
       </c>
       <c r="B18" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="C18">
         <v>202</v>
@@ -3381,7 +3349,7 @@
         <v>118</v>
       </c>
       <c r="B19" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="C19">
         <v>294</v>
@@ -3407,7 +3375,7 @@
         <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="C20">
         <v>81</v>
@@ -3433,7 +3401,7 @@
         <v>120</v>
       </c>
       <c r="B21" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="C21">
         <v>115</v>
@@ -3459,7 +3427,7 @@
         <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="C22">
         <v>112</v>
@@ -3485,7 +3453,7 @@
         <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="C23">
         <v>83</v>
@@ -3511,7 +3479,7 @@
         <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="C24">
         <v>118</v>
@@ -3537,7 +3505,7 @@
         <v>124</v>
       </c>
       <c r="B25" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="C25">
         <v>117</v>
@@ -3563,7 +3531,7 @@
         <v>125</v>
       </c>
       <c r="B26" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="C26">
         <v>87</v>
@@ -3589,7 +3557,7 @@
         <v>126</v>
       </c>
       <c r="B27" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="C27">
         <v>125</v>
@@ -3615,7 +3583,7 @@
         <v>127</v>
       </c>
       <c r="B28" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="C28">
         <v>123</v>
@@ -3641,7 +3609,7 @@
         <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="C29">
         <v>88</v>
@@ -3667,7 +3635,7 @@
         <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="C30">
         <v>127</v>
@@ -3693,7 +3661,7 @@
         <v>130</v>
       </c>
       <c r="B31" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="C31">
         <v>127</v>
@@ -3719,7 +3687,7 @@
         <v>132</v>
       </c>
       <c r="B32" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="C32">
         <v>172</v>
@@ -3745,7 +3713,7 @@
         <v>133</v>
       </c>
       <c r="B33" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="C33">
         <v>218</v>
@@ -3771,7 +3739,7 @@
         <v>134</v>
       </c>
       <c r="B34" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="C34">
         <v>102</v>
@@ -3797,7 +3765,7 @@
         <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="C35">
         <v>83</v>
@@ -3823,7 +3791,7 @@
         <v>201</v>
       </c>
       <c r="B36" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="C36">
         <v>401</v>
@@ -3837,7 +3805,7 @@
         <v>202</v>
       </c>
       <c r="B37" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="C37">
         <v>114</v>
@@ -3863,7 +3831,7 @@
         <v>203</v>
       </c>
       <c r="B38" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="C38">
         <v>84</v>
@@ -3889,7 +3857,7 @@
         <v>204</v>
       </c>
       <c r="B39" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="C39">
         <v>81</v>
@@ -3915,7 +3883,7 @@
         <v>205</v>
       </c>
       <c r="B40" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="C40">
         <v>118</v>
@@ -3941,7 +3909,7 @@
         <v>206</v>
       </c>
       <c r="B41" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="C41">
         <v>120</v>
@@ -3967,7 +3935,7 @@
         <v>207</v>
       </c>
       <c r="B42" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="C42">
         <v>89</v>
@@ -3993,7 +3961,7 @@
         <v>208</v>
       </c>
       <c r="B43" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="C43">
         <v>84</v>
@@ -4019,7 +3987,7 @@
         <v>209</v>
       </c>
       <c r="B44" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="C44">
         <v>124</v>
@@ -4045,7 +4013,7 @@
         <v>210</v>
       </c>
       <c r="B45" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="C45">
         <v>126</v>
@@ -4071,7 +4039,7 @@
         <v>211</v>
       </c>
       <c r="B46" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="C46">
         <v>91</v>
@@ -4097,7 +4065,7 @@
         <v>212</v>
       </c>
       <c r="B47" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="C47">
         <v>88</v>
@@ -4123,7 +4091,7 @@
         <v>213</v>
       </c>
       <c r="B48" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="C48">
         <v>131</v>
@@ -4149,7 +4117,7 @@
         <v>214</v>
       </c>
       <c r="B49" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="C49">
         <v>130</v>
@@ -4175,7 +4143,7 @@
         <v>215</v>
       </c>
       <c r="B50" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="C50">
         <v>93</v>
@@ -4201,7 +4169,7 @@
         <v>216</v>
       </c>
       <c r="B51" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="C51">
         <v>59</v>
@@ -4227,7 +4195,7 @@
         <v>217</v>
       </c>
       <c r="B52" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="C52">
         <v>166</v>
@@ -4253,7 +4221,7 @@
         <v>218</v>
       </c>
       <c r="B53" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="C53">
         <v>186</v>
@@ -4279,7 +4247,7 @@
         <v>219</v>
       </c>
       <c r="B54" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="C54">
         <v>61</v>
@@ -4305,7 +4273,7 @@
         <v>220</v>
       </c>
       <c r="B55" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="C55">
         <v>171</v>
@@ -4331,7 +4299,7 @@
         <v>221</v>
       </c>
       <c r="B56" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="C56">
         <v>178</v>
@@ -4357,7 +4325,7 @@
         <v>222</v>
       </c>
       <c r="B57" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="C57">
         <v>62</v>
@@ -4383,7 +4351,7 @@
         <v>223</v>
       </c>
       <c r="B58" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="C58">
         <v>174</v>
@@ -4409,7 +4377,7 @@
         <v>224</v>
       </c>
       <c r="B59" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="C59">
         <v>181</v>
@@ -4435,7 +4403,7 @@
         <v>225</v>
       </c>
       <c r="B60" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="C60" s="8">
         <v>197</v>
@@ -4469,7 +4437,7 @@
         <v>301</v>
       </c>
       <c r="B61" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="C61">
         <v>169</v>
@@ -4489,7 +4457,7 @@
         <v>302</v>
       </c>
       <c r="B62" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="C62">
         <v>158</v>
@@ -4509,7 +4477,7 @@
         <v>303</v>
       </c>
       <c r="B63" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="C63">
         <v>71</v>
@@ -4529,7 +4497,7 @@
         <v>305</v>
       </c>
       <c r="B64" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="C64">
         <v>134</v>
@@ -4552,7 +4520,7 @@
         <v>306</v>
       </c>
       <c r="B65" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="C65">
         <v>147</v>
@@ -4575,7 +4543,7 @@
         <v>307</v>
       </c>
       <c r="B66" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="C66">
         <v>155</v>
@@ -4598,7 +4566,7 @@
         <v>308</v>
       </c>
       <c r="B67" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="C67" s="8">
         <v>75</v>
@@ -4630,7 +4598,7 @@
         <v>310</v>
       </c>
       <c r="B68" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="C68">
         <v>52</v>
@@ -4653,7 +4621,7 @@
         <v>311</v>
       </c>
       <c r="B69" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="C69">
         <v>193</v>
@@ -4676,7 +4644,7 @@
         <v>312</v>
       </c>
       <c r="B70" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="C70">
         <v>133</v>
@@ -4699,7 +4667,7 @@
         <v>313</v>
       </c>
       <c r="B71" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="C71">
         <v>72</v>
@@ -4719,7 +4687,7 @@
         <v>314</v>
       </c>
       <c r="B72" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="C72">
         <v>79</v>
@@ -4739,7 +4707,7 @@
         <v>315</v>
       </c>
       <c r="B73" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="C73">
         <v>85</v>
@@ -4762,7 +4730,7 @@
         <v>316</v>
       </c>
       <c r="B74" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="C74">
         <v>90</v>
@@ -4785,7 +4753,7 @@
         <v>401</v>
       </c>
       <c r="B75" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="C75">
         <v>7</v>
@@ -4805,7 +4773,7 @@
         <v>402</v>
       </c>
       <c r="B76" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="C76">
         <v>7</v>
@@ -4825,7 +4793,7 @@
         <v>403</v>
       </c>
       <c r="B77" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C77">
         <v>7</v>
@@ -4845,7 +4813,7 @@
         <v>404</v>
       </c>
       <c r="B78" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="C78">
         <v>7</v>
@@ -4865,7 +4833,7 @@
         <v>405</v>
       </c>
       <c r="B79" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C79">
         <v>7</v>
@@ -4885,7 +4853,7 @@
         <v>406</v>
       </c>
       <c r="B80" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="C80">
         <v>7</v>
@@ -4905,7 +4873,7 @@
         <v>407</v>
       </c>
       <c r="B81" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="C81">
         <v>7</v>
@@ -4925,7 +4893,7 @@
         <v>408</v>
       </c>
       <c r="B82" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="C82">
         <v>7</v>
@@ -4945,7 +4913,7 @@
         <v>409</v>
       </c>
       <c r="B83" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="C83">
         <v>7</v>
@@ -4965,7 +4933,7 @@
         <v>410</v>
       </c>
       <c r="B84" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="C84">
         <v>7</v>
@@ -4985,7 +4953,7 @@
         <v>411</v>
       </c>
       <c r="B85" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C85">
         <v>7</v>
@@ -5005,7 +4973,7 @@
         <v>412</v>
       </c>
       <c r="B86" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="C86">
         <v>7</v>
@@ -5025,7 +4993,7 @@
         <v>413</v>
       </c>
       <c r="B87" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="C87">
         <v>7</v>
@@ -5045,7 +5013,7 @@
         <v>414</v>
       </c>
       <c r="B88" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C88">
         <v>7</v>
@@ -5065,7 +5033,7 @@
         <v>415</v>
       </c>
       <c r="B89" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="C89">
         <v>7</v>
@@ -5085,7 +5053,7 @@
         <v>416</v>
       </c>
       <c r="B90" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C90">
         <v>7</v>
@@ -5105,7 +5073,7 @@
         <v>417</v>
       </c>
       <c r="B91" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="C91">
         <v>7</v>
@@ -5125,7 +5093,7 @@
         <v>418</v>
       </c>
       <c r="B92" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="C92">
         <v>7</v>
@@ -5145,7 +5113,7 @@
         <v>419</v>
       </c>
       <c r="B93" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C93">
         <v>7</v>
@@ -5165,7 +5133,7 @@
         <v>420</v>
       </c>
       <c r="B94" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C94">
         <v>7</v>
@@ -5185,7 +5153,7 @@
         <v>421</v>
       </c>
       <c r="B95" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="C95">
         <v>7</v>
@@ -5205,7 +5173,7 @@
         <v>422</v>
       </c>
       <c r="B96" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="C96">
         <v>7</v>
@@ -5225,7 +5193,7 @@
         <v>423</v>
       </c>
       <c r="B97" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="C97">
         <v>7</v>
@@ -5245,7 +5213,7 @@
         <v>424</v>
       </c>
       <c r="B98" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="C98">
         <v>7</v>
@@ -5265,7 +5233,7 @@
         <v>425</v>
       </c>
       <c r="B99" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="C99">
         <v>7</v>
@@ -5285,7 +5253,7 @@
         <v>426</v>
       </c>
       <c r="B100" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="C100">
         <v>7</v>
@@ -5305,7 +5273,7 @@
         <v>427</v>
       </c>
       <c r="B101" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C101">
         <v>7</v>
@@ -5325,7 +5293,7 @@
         <v>428</v>
       </c>
       <c r="B102" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="C102">
         <v>7</v>
@@ -5345,7 +5313,7 @@
         <v>429</v>
       </c>
       <c r="B103" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="C103">
         <v>7</v>
@@ -5365,7 +5333,7 @@
         <v>430</v>
       </c>
       <c r="B104" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="C104">
         <v>7</v>
@@ -5385,7 +5353,7 @@
         <v>431</v>
       </c>
       <c r="B105" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C105">
         <v>7</v>
@@ -5405,7 +5373,7 @@
         <v>432</v>
       </c>
       <c r="B106" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C106">
         <v>7</v>
@@ -5425,7 +5393,7 @@
         <v>433</v>
       </c>
       <c r="B107" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="C107">
         <v>7</v>
@@ -5445,7 +5413,7 @@
         <v>434</v>
       </c>
       <c r="B108" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="C108">
         <v>7</v>
@@ -5465,7 +5433,7 @@
         <v>435</v>
       </c>
       <c r="B109" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="C109">
         <v>7</v>
@@ -5485,7 +5453,7 @@
         <v>436</v>
       </c>
       <c r="B110" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C110">
         <v>7</v>
@@ -5505,7 +5473,7 @@
         <v>437</v>
       </c>
       <c r="B111" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="C111">
         <v>7</v>
@@ -5525,7 +5493,7 @@
         <v>438</v>
       </c>
       <c r="B112" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="C112">
         <v>7</v>
@@ -5545,7 +5513,7 @@
         <v>439</v>
       </c>
       <c r="B113" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="C113">
         <v>7</v>
@@ -5565,7 +5533,7 @@
         <v>440</v>
       </c>
       <c r="B114" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C114">
         <v>7</v>
@@ -5585,7 +5553,7 @@
         <v>441</v>
       </c>
       <c r="B115" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="C115">
         <v>7</v>
@@ -5605,7 +5573,7 @@
         <v>442</v>
       </c>
       <c r="B116" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="C116">
         <v>7</v>
@@ -5625,7 +5593,7 @@
         <v>443</v>
       </c>
       <c r="B117" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="C117">
         <v>7</v>
@@ -5645,7 +5613,7 @@
         <v>444</v>
       </c>
       <c r="B118" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="C118">
         <v>7</v>
@@ -5665,7 +5633,7 @@
         <v>445</v>
       </c>
       <c r="B119" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C119">
         <v>7</v>
@@ -5685,7 +5653,7 @@
         <v>446</v>
       </c>
       <c r="B120" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="C120">
         <v>7</v>
@@ -5705,7 +5673,7 @@
         <v>447</v>
       </c>
       <c r="B121" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="C121">
         <v>7</v>
@@ -5725,7 +5693,7 @@
         <v>448</v>
       </c>
       <c r="B122" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C122">
         <v>7</v>
@@ -5745,7 +5713,7 @@
         <v>449</v>
       </c>
       <c r="B123" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="C123">
         <v>7</v>
@@ -5765,7 +5733,7 @@
         <v>450</v>
       </c>
       <c r="B124" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C124">
         <v>7</v>
@@ -5785,7 +5753,7 @@
         <v>451</v>
       </c>
       <c r="B125" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="C125">
         <v>7</v>
@@ -5805,7 +5773,7 @@
         <v>452</v>
       </c>
       <c r="B126" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C126">
         <v>7</v>
@@ -5825,7 +5793,7 @@
         <v>453</v>
       </c>
       <c r="B127" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="C127">
         <v>7</v>
@@ -5845,7 +5813,7 @@
         <v>454</v>
       </c>
       <c r="B128" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="C128">
         <v>7</v>
@@ -5865,7 +5833,7 @@
         <v>455</v>
       </c>
       <c r="B129" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="C129">
         <v>7</v>
@@ -5885,7 +5853,7 @@
         <v>456</v>
       </c>
       <c r="B130" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="C130">
         <v>7</v>
@@ -5905,7 +5873,7 @@
         <v>457</v>
       </c>
       <c r="B131" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="C131">
         <v>7</v>
@@ -5925,7 +5893,7 @@
         <v>458</v>
       </c>
       <c r="B132" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="C132">
         <v>7</v>
@@ -5945,7 +5913,7 @@
         <v>459</v>
       </c>
       <c r="B133" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="C133">
         <v>7</v>
@@ -5965,7 +5933,7 @@
         <v>460</v>
       </c>
       <c r="B134" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="C134">
         <v>7</v>
@@ -5985,7 +5953,7 @@
         <v>461</v>
       </c>
       <c r="B135" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="C135">
         <v>7</v>
@@ -6005,7 +5973,7 @@
         <v>462</v>
       </c>
       <c r="B136" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="C136">
         <v>7</v>
@@ -6025,7 +5993,7 @@
         <v>463</v>
       </c>
       <c r="B137" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="C137">
         <v>7</v>
@@ -6045,7 +6013,7 @@
         <v>464</v>
       </c>
       <c r="B138" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="C138">
         <v>7</v>
@@ -6065,7 +6033,7 @@
         <v>465</v>
       </c>
       <c r="B139" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="C139">
         <v>7</v>
@@ -6085,7 +6053,7 @@
         <v>466</v>
       </c>
       <c r="B140" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="C140">
         <v>7</v>
@@ -6105,7 +6073,7 @@
         <v>467</v>
       </c>
       <c r="B141" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="C141">
         <v>7</v>
@@ -6125,7 +6093,7 @@
         <v>468</v>
       </c>
       <c r="B142" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="C142">
         <v>7</v>
@@ -6145,7 +6113,7 @@
         <v>469</v>
       </c>
       <c r="B143" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="C143">
         <v>7</v>
@@ -6165,7 +6133,7 @@
         <v>470</v>
       </c>
       <c r="B144" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="C144">
         <v>7</v>
@@ -6185,7 +6153,7 @@
         <v>471</v>
       </c>
       <c r="B145" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="C145">
         <v>7</v>
@@ -6205,7 +6173,7 @@
         <v>472</v>
       </c>
       <c r="B146" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="C146">
         <v>7</v>
@@ -6225,7 +6193,7 @@
         <v>473</v>
       </c>
       <c r="B147" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="C147">
         <v>7</v>
@@ -6245,7 +6213,7 @@
         <v>474</v>
       </c>
       <c r="B148" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="C148">
         <v>7</v>
@@ -6265,7 +6233,7 @@
         <v>475</v>
       </c>
       <c r="B149" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="C149">
         <v>7</v>
@@ -6285,7 +6253,7 @@
         <v>476</v>
       </c>
       <c r="B150" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="C150">
         <v>7</v>
@@ -6305,7 +6273,7 @@
         <v>477</v>
       </c>
       <c r="B151" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="C151">
         <v>7</v>
@@ -6325,7 +6293,7 @@
         <v>478</v>
       </c>
       <c r="B152" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="C152">
         <v>7</v>
@@ -6345,7 +6313,7 @@
         <v>479</v>
       </c>
       <c r="B153" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="C153">
         <v>7</v>
@@ -6365,7 +6333,7 @@
         <v>480</v>
       </c>
       <c r="B154" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="C154">
         <v>7</v>
@@ -6385,7 +6353,7 @@
         <v>481</v>
       </c>
       <c r="B155" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="C155">
         <v>7</v>
@@ -6405,7 +6373,7 @@
         <v>482</v>
       </c>
       <c r="B156" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="C156">
         <v>7</v>
@@ -6425,7 +6393,7 @@
         <v>483</v>
       </c>
       <c r="B157" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="C157">
         <v>7</v>
@@ -6445,7 +6413,7 @@
         <v>484</v>
       </c>
       <c r="B158" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="C158">
         <v>7</v>
@@ -6465,7 +6433,7 @@
         <v>485</v>
       </c>
       <c r="B159" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="C159">
         <v>7</v>
@@ -6485,7 +6453,7 @@
         <v>486</v>
       </c>
       <c r="B160" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="C160">
         <v>7</v>
@@ -6505,7 +6473,7 @@
         <v>487</v>
       </c>
       <c r="B161" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="C161">
         <v>7</v>
@@ -6525,7 +6493,7 @@
         <v>488</v>
       </c>
       <c r="B162" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="C162">
         <v>7</v>
@@ -6545,7 +6513,7 @@
         <v>489</v>
       </c>
       <c r="B163" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="C163">
         <v>7</v>
@@ -6565,7 +6533,7 @@
         <v>490</v>
       </c>
       <c r="B164" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="C164">
         <v>7</v>
@@ -6585,7 +6553,7 @@
         <v>491</v>
       </c>
       <c r="B165" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="C165">
         <v>7</v>
@@ -6605,7 +6573,7 @@
         <v>492</v>
       </c>
       <c r="B166" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="C166">
         <v>7</v>
@@ -6625,7 +6593,7 @@
         <v>493</v>
       </c>
       <c r="B167" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="C167">
         <v>7</v>
@@ -6645,7 +6613,7 @@
         <v>494</v>
       </c>
       <c r="B168" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="C168">
         <v>7</v>
@@ -6665,7 +6633,7 @@
         <v>495</v>
       </c>
       <c r="B169" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="C169">
         <v>7</v>
@@ -6685,7 +6653,7 @@
         <v>496</v>
       </c>
       <c r="B170" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="C170">
         <v>7</v>
@@ -6705,7 +6673,7 @@
         <v>497</v>
       </c>
       <c r="B171" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="C171">
         <v>7</v>
@@ -6725,7 +6693,7 @@
         <v>498</v>
       </c>
       <c r="B172" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="C172">
         <v>7</v>
@@ -6745,7 +6713,7 @@
         <v>499</v>
       </c>
       <c r="B173" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
       <c r="C173">
         <v>7</v>
@@ -6765,7 +6733,7 @@
         <v>500</v>
       </c>
       <c r="B174" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="C174">
         <v>7</v>
@@ -6785,7 +6753,7 @@
         <v>501</v>
       </c>
       <c r="B175" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="C175">
         <v>7</v>
@@ -6805,7 +6773,7 @@
         <v>502</v>
       </c>
       <c r="B176" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="C176">
         <v>1</v>
@@ -6823,7 +6791,7 @@
         <v>503</v>
       </c>
       <c r="B177" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="C177">
         <v>1</v>
@@ -6841,7 +6809,7 @@
         <v>504</v>
       </c>
       <c r="B178" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="C178">
         <v>1</v>
@@ -6859,7 +6827,7 @@
         <v>505</v>
       </c>
       <c r="B179" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -6877,7 +6845,7 @@
         <v>506</v>
       </c>
       <c r="B180" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="C180">
         <v>7</v>
@@ -6905,8 +6873,8 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.140625" customWidth="1"/>
     <col min="2" max="2" width="66.5703125" style="2" customWidth="1"/>
@@ -6915,7 +6883,7 @@
     <col min="5" max="5" width="11.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="71.5703125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="98.85546875" style="2" customWidth="1"/>
     <col min="9" max="9" width="48.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6927,7 +6895,7 @@
         <v>93</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D1" t="s">
         <v>92</v>
@@ -6945,7 +6913,7 @@
         <v>136</v>
       </c>
       <c r="I1" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -6966,738 +6934,722 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>170</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>71</v>
+        <v>113</v>
       </c>
       <c r="D3" t="s">
-        <v>178</v>
+        <v>10</v>
       </c>
       <c r="E3" s="4">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G3" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>169</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>178</v>
+        <v>11</v>
       </c>
       <c r="E4" s="4">
-        <v>10000</v>
+        <v>2460</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G4" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>10000</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>170</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>182</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>178</v>
+        <v>27</v>
       </c>
       <c r="E5" s="4">
-        <v>1940</v>
+        <v>1051.2</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G5" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>1940</v>
+        <v>1051.2</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>172</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>169</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>116</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
       </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="E6" s="4">
-        <v>18000</v>
+        <v>748.15</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G6" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>18000</v>
+        <v>748.15</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="I6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>170</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>71</v>
+        <v>115</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>178</v>
+        <v>6</v>
       </c>
       <c r="E7" s="4">
-        <v>5710</v>
+        <v>6096.65</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G7" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>5710</v>
+        <v>6096.65</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>173</v>
+        <v>100</v>
+      </c>
+      <c r="I7" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>169</v>
+        <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>70</v>
+        <v>114</v>
+      </c>
+      <c r="C8" t="s">
+        <v>65</v>
       </c>
       <c r="D8" t="s">
-        <v>178</v>
+        <v>7</v>
       </c>
       <c r="E8" s="4">
-        <v>20000</v>
+        <v>7502.9</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G8" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>20000</v>
+        <v>7502.9</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>170</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>71</v>
+        <v>126</v>
+      </c>
+      <c r="C9" t="s">
+        <v>72</v>
       </c>
       <c r="D9" t="s">
-        <v>178</v>
+        <v>80</v>
       </c>
       <c r="E9" s="4">
-        <v>10770</v>
+        <f>16750</f>
+        <v>16750</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G9" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>10770</v>
+        <v>16750</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>169</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>70</v>
+        <v>187</v>
+      </c>
+      <c r="C10" t="s">
+        <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>178</v>
+        <v>80</v>
       </c>
       <c r="E10" s="4">
-        <v>25000</v>
+        <f>887</f>
+        <v>887</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G10" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>25000</v>
+        <v>887</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>113</v>
+        <v>128</v>
+      </c>
+      <c r="C11" t="s">
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="4">
-        <v>3000</v>
+        <v>22</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G11" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3000</v>
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>112</v>
+        <v>127</v>
+      </c>
+      <c r="C12" t="s">
+        <v>72</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="4">
-        <v>2460</v>
+        <v>21</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G12" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2460</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>119</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="E13" s="4">
-        <v>1051.2</v>
+        <f>1140*12</f>
+        <v>13680</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G13" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>1051.2</v>
+        <v>13680</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>28</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="E14" s="4">
-        <v>748.15</v>
+        <f>2836.8*12</f>
+        <v>34041.600000000006</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G14" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>748.15</v>
+        <v>34041.600000000006</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="I14" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>105</v>
       </c>
       <c r="E15" s="4">
-        <v>6096.65</v>
+        <f>1518*12</f>
+        <v>18216</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G15" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>6096.65</v>
+        <v>18216</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I15" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="E16" s="4">
-        <v>7502.9</v>
+        <v>516</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G16" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>7502.9</v>
+        <v>516</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="E17" s="4">
-        <f>16750</f>
-        <v>16750</v>
+        <v>456</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G17" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>16750</v>
+        <v>456</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="165" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>199</v>
+        <v>125</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="E18" s="4">
-        <f>887</f>
-        <v>887</v>
+        <v>660</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G18" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>887</v>
+        <v>660</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>128</v>
+        <v>189</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>190</v>
+      </c>
+      <c r="E19" s="4">
+        <v>434.5</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G19" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>0</v>
-      </c>
-      <c r="H19" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>434.5</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C20" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>21</v>
+        <v>79</v>
+      </c>
+      <c r="E20" s="4">
+        <v>2400</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" t="s">
-        <v>132</v>
+        <v>2880</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I20" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>119</v>
+        <v>140</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="D21" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="E21" s="4">
-        <f>1140*12</f>
-        <v>13680</v>
+        <v>2400</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>13680</v>
+        <v>2880</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>102</v>
+        <v>133</v>
+      </c>
+      <c r="I21" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="E22" s="4">
-        <f>2836.8*12</f>
-        <v>34041.600000000006</v>
+        <v>2450</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>34041.600000000006</v>
+        <v>2940</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>103</v>
+        <v>133</v>
+      </c>
+      <c r="I22" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="D23" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="E23" s="4">
-        <f>1518*12</f>
-        <v>18216</v>
+        <v>2200</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>18216</v>
+        <v>2640</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="I23" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C24" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>26</v>
       </c>
       <c r="E24" s="4">
-        <v>516</v>
+        <v>160</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G24" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>516</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E25" s="4">
-        <v>456</v>
+        <f>2400*12</f>
+        <v>28800</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G25" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>456</v>
+        <v>28800</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="225" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="E26" s="4">
-        <v>660</v>
+        <f>1320*12</f>
+        <v>15840</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G26" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>660</v>
+        <v>15840</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C27" t="s">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="D27" t="s">
-        <v>202</v>
+        <v>17</v>
       </c>
       <c r="E27" s="4">
-        <v>434.5</v>
+        <v>3198.13</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>2</v>
       </c>
       <c r="G27" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>434.5</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>200</v>
+        <v>3198.13</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C28" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="E28" s="4">
-        <v>2400</v>
+        <v>3322.8</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2880</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I28" t="s">
-        <v>200</v>
+        <v>3322.8</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C29" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E29" s="4">
-        <v>2400</v>
+        <v>3138.27</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2880</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I29" t="s">
-        <v>200</v>
+        <v>3138.27</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -7705,29 +7657,26 @@
         <v>13</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D30" t="s">
         <v>79</v>
       </c>
       <c r="E30" s="4">
-        <v>2450</v>
+        <v>240</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>1</v>
       </c>
       <c r="G30" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2940</v>
+        <v>288</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="I30" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -7735,385 +7684,188 @@
         <v>13</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C31" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D31" t="s">
         <v>79</v>
       </c>
       <c r="E31" s="4">
-        <v>2200</v>
+        <v>240</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>1</v>
       </c>
       <c r="G31" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>2640</v>
+        <v>288</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I31" t="s">
-        <v>200</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>25</v>
+        <v>141</v>
+      </c>
+      <c r="C32" t="s">
+        <v>87</v>
       </c>
       <c r="D32" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="E32" s="4">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>160</v>
+        <v>288</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="D33" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="E33" s="4">
-        <f>2400*12</f>
-        <v>28800</v>
+        <v>240</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="4">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>28800</v>
+        <v>288</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>12</v>
+        <v>98</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" t="s">
-        <v>55</v>
+        <v>171</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="D34" t="s">
-        <v>108</v>
-      </c>
-      <c r="E34" s="4">
-        <f>1320*12</f>
-        <v>15840</v>
-      </c>
-      <c r="F34" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E34" s="5">
+        <v>10000</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G34" s="4">
+      <c r="G34" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>15840</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>106</v>
-      </c>
+        <v>10000</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>122</v>
+        <v>173</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
-      </c>
-      <c r="E35" s="4">
-        <v>3198.13</v>
-      </c>
-      <c r="F35" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E35" s="5">
+        <v>12500</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G35" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3198.13</v>
-      </c>
+        <v>12500</v>
+      </c>
+      <c r="H35" s="3"/>
+      <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>121</v>
+        <v>172</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="D36" t="s">
-        <v>16</v>
-      </c>
-      <c r="E36" s="4">
-        <v>3322.8</v>
-      </c>
-      <c r="F36" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E36" s="5">
+        <v>15000</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3322.8</v>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="H36" s="3"/>
+      <c r="I36" s="2"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>120</v>
+        <v>98</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="D37" t="s">
-        <v>15</v>
-      </c>
-      <c r="E37" s="4">
-        <v>3138.27</v>
-      </c>
-      <c r="F37" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E37" s="5">
+        <v>16800</v>
+      </c>
+      <c r="F37" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G37" s="4">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>3138.27</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C38" t="s">
-        <v>85</v>
-      </c>
-      <c r="D38" t="s">
-        <v>79</v>
-      </c>
-      <c r="E38" s="4">
-        <v>240</v>
-      </c>
-      <c r="F38" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="G38" s="4">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>288</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C39" t="s">
-        <v>86</v>
-      </c>
-      <c r="D39" t="s">
-        <v>79</v>
-      </c>
-      <c r="E39" s="4">
-        <v>240</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="G39" s="4">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>288</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C40" t="s">
-        <v>87</v>
-      </c>
-      <c r="D40" t="s">
-        <v>79</v>
-      </c>
-      <c r="E40" s="4">
-        <v>240</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="G40" s="4">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>288</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C41" t="s">
-        <v>88</v>
-      </c>
-      <c r="D41" t="s">
-        <v>79</v>
-      </c>
-      <c r="E41" s="4">
-        <v>240</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="G41" s="4">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>288</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D42" t="s">
-        <v>178</v>
-      </c>
-      <c r="E42" s="5">
-        <v>10000</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G42" s="5">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>10000</v>
-      </c>
-      <c r="H42" s="3"/>
-      <c r="I42" s="2"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D43" t="s">
-        <v>178</v>
-      </c>
-      <c r="E43" s="5">
-        <v>12500</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G43" s="5">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>12500</v>
-      </c>
-      <c r="H43" s="3"/>
-      <c r="I43" s="2"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D44" t="s">
-        <v>178</v>
-      </c>
-      <c r="E44" s="5">
-        <v>15000</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G44" s="5">
-        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
-        <v>15000</v>
-      </c>
-      <c r="H44" s="3"/>
-      <c r="I44" s="2"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D45" t="s">
-        <v>27</v>
-      </c>
-      <c r="E45" s="5">
-        <v>16800</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G45" s="5">
+      <c r="G37" s="5">
         <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
         <v>16800</v>
       </c>
-      <c r="H45" s="3" t="s">
+      <c r="H37" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>200</v>
+      <c r="I37" s="2" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -8142,7 +7894,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -8151,18 +7903,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="B1" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C1" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B2">
         <f>5735*2.5</f>
@@ -8186,7 +7938,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
@@ -8202,39 +7954,39 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="B1" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>411</v>
+        <v>398</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>412</v>
+        <v>399</v>
       </c>
       <c r="G1" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="H1" t="s">
         <v>136</v>
       </c>
       <c r="I1" t="s">
-        <v>415</v>
+        <v>402</v>
       </c>
       <c r="J1" t="s">
-        <v>414</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>70</v>
@@ -8244,7 +7996,7 @@
         <v>9.6000000000000002E-2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="E2" s="1">
         <v>392</v>
@@ -8256,7 +8008,7 @@
         <v>120</v>
       </c>
       <c r="H2" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="I2" s="13">
         <v>0.3</v>
@@ -8267,7 +8019,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
@@ -8276,7 +8028,7 @@
         <v>0.12559999999999999</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="E3" s="1">
         <v>0.12559999999999999</v>
@@ -8288,7 +8040,7 @@
         <v>140</v>
       </c>
       <c r="H3" t="s">
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="I3" s="13">
         <v>0.08</v>

</xml_diff>

<commit_message>
Ajout perte de chaleur ECS
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1352" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABBA670F-8EBD-46A0-88D7-23996C8CEBB2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -1366,82 +1366,6 @@
     <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="31">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1775,6 +1699,82 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1788,10 +1788,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}" name="Provisions" displayName="Provisions" ref="A1:F35">
   <autoFilter ref="A1:F35" xr:uid="{13C2BCD2-5CEA-4301-A571-688E40226767}"/>
@@ -1803,8 +1799,8 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29" dataCellStyle="Monétaire"/>
-    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="25" totalsRowDxfId="24" dataCellStyle="Monétaire"/>
+    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1817,24 +1813,24 @@
     <sortCondition ref="A1:A180"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="22"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="26">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="21">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="18"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="17"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="16"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="15"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="17"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="16"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="13"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="12"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="11"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="10"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1847,17 +1843,17 @@
     <sortCondition ref="B1:B37"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="2">
       <calculatedColumnFormula>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1884,13 +1880,13 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
-    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix TTC de l'unité" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix TTC de l'unité" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="27"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
-    <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (kW)" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (kW)" dataDxfId="26"/>
     <tableColumn id="11" xr3:uid="{D0B5F61C-1D85-4C5E-A117-B774F88FE50E}" name="Seuil de durée d'activation (mn)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -7292,7 +7288,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -7319,7 +7315,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -7346,7 +7342,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>

</xml_diff>